<commit_message>
adjust tenancy period display
</commit_message>
<xml_diff>
--- a/building_tenants_test_data.xlsx
+++ b/building_tenants_test_data.xlsx
@@ -466,10 +466,10 @@
         <v>942</v>
       </c>
       <c r="H2" t="str">
-        <v>2025-05-01</v>
+        <v>2025</v>
       </c>
       <c r="I2" t="str">
-        <v>2026-05-31</v>
+        <v>2026</v>
       </c>
       <c r="J2" t="str">
         <v>Current</v>
@@ -498,10 +498,10 @@
         <v>972.75</v>
       </c>
       <c r="H3" t="str">
-        <v>2025-06-01</v>
+        <v>2025</v>
       </c>
       <c r="I3" t="str">
-        <v>2026-06-31</v>
+        <v>2026</v>
       </c>
       <c r="J3" t="str">
         <v>Notice</v>
@@ -530,10 +530,10 @@
         <v>1003.5</v>
       </c>
       <c r="H4" t="str">
-        <v>2025-07-01</v>
+        <v>2025</v>
       </c>
       <c r="I4" t="str">
-        <v>2026-07-31</v>
+        <v>2026</v>
       </c>
       <c r="J4" t="str">
         <v>Current</v>
@@ -562,10 +562,10 @@
         <v>1034.25</v>
       </c>
       <c r="H5" t="str">
-        <v>2025-08-01</v>
+        <v>2025</v>
       </c>
       <c r="I5" t="str">
-        <v>2026-08-31</v>
+        <v>2026</v>
       </c>
       <c r="J5" t="str">
         <v>Current</v>
@@ -594,10 +594,10 @@
         <v>942</v>
       </c>
       <c r="H6" t="str">
-        <v>2025-05-01</v>
+        <v>2025</v>
       </c>
       <c r="I6" t="str">
-        <v>2026-05-31</v>
+        <v>2026</v>
       </c>
       <c r="J6" t="str">
         <v>Current</v>
@@ -626,10 +626,10 @@
         <v>972.75</v>
       </c>
       <c r="H7" t="str">
-        <v>2025-06-01</v>
+        <v>2025</v>
       </c>
       <c r="I7" t="str">
-        <v>2026-06-31</v>
+        <v>2026</v>
       </c>
       <c r="J7" t="str">
         <v>Current</v>
@@ -658,10 +658,10 @@
         <v>1003.5</v>
       </c>
       <c r="H8" t="str">
-        <v>2025-07-01</v>
+        <v>2025</v>
       </c>
       <c r="I8" t="str">
-        <v>2026-07-31</v>
+        <v>2026</v>
       </c>
       <c r="J8" t="str">
         <v>Current</v>
@@ -690,10 +690,10 @@
         <v>1034.25</v>
       </c>
       <c r="H9" t="str">
-        <v>2025-08-01</v>
+        <v>2025</v>
       </c>
       <c r="I9" t="str">
-        <v>2026-08-31</v>
+        <v>2026</v>
       </c>
       <c r="J9" t="str">
         <v>Current</v>
@@ -722,10 +722,10 @@
         <v>1065</v>
       </c>
       <c r="H10" t="str">
-        <v>2025-09-01</v>
+        <v>2025</v>
       </c>
       <c r="I10" t="str">
-        <v>2026-09-31</v>
+        <v>2026</v>
       </c>
       <c r="J10" t="str">
         <v>Current</v>
@@ -754,10 +754,10 @@
         <v>942</v>
       </c>
       <c r="H11" t="str">
-        <v>2025-05-01</v>
+        <v>2025</v>
       </c>
       <c r="I11" t="str">
-        <v>2026-05-31</v>
+        <v>2026</v>
       </c>
       <c r="J11" t="str">
         <v>Current</v>
@@ -786,10 +786,10 @@
         <v>972.75</v>
       </c>
       <c r="H12" t="str">
-        <v>2025-06-01</v>
+        <v>2025</v>
       </c>
       <c r="I12" t="str">
-        <v>2026-06-31</v>
+        <v>2026</v>
       </c>
       <c r="J12" t="str">
         <v>Current</v>
@@ -818,10 +818,10 @@
         <v>942</v>
       </c>
       <c r="H13" t="str">
-        <v>2025-05-01</v>
+        <v>2025</v>
       </c>
       <c r="I13" t="str">
-        <v>2026-05-31</v>
+        <v>2026</v>
       </c>
       <c r="J13" t="str">
         <v>Current</v>
@@ -850,10 +850,10 @@
         <v>972.75</v>
       </c>
       <c r="H14" t="str">
-        <v>2025-06-01</v>
+        <v>2025</v>
       </c>
       <c r="I14" t="str">
-        <v>2026-06-31</v>
+        <v>2026</v>
       </c>
       <c r="J14" t="str">
         <v>Notice</v>
@@ -882,10 +882,10 @@
         <v>1003.5</v>
       </c>
       <c r="H15" t="str">
-        <v>2025-07-01</v>
+        <v>2025</v>
       </c>
       <c r="I15" t="str">
-        <v>2026-07-31</v>
+        <v>2026</v>
       </c>
       <c r="J15" t="str">
         <v>Current</v>
@@ -914,10 +914,10 @@
         <v>1034.25</v>
       </c>
       <c r="H16" t="str">
-        <v>2025-08-01</v>
+        <v>2025</v>
       </c>
       <c r="I16" t="str">
-        <v>2026-08-31</v>
+        <v>2026</v>
       </c>
       <c r="J16" t="str">
         <v>Current</v>
@@ -946,10 +946,10 @@
         <v>1065</v>
       </c>
       <c r="H17" t="str">
-        <v>2025-09-01</v>
+        <v>2025</v>
       </c>
       <c r="I17" t="str">
-        <v>2026-09-31</v>
+        <v>2026</v>
       </c>
       <c r="J17" t="str">
         <v>Current</v>
@@ -978,10 +978,10 @@
         <v>942</v>
       </c>
       <c r="H18" t="str">
-        <v>2025-05-01</v>
+        <v>2025</v>
       </c>
       <c r="I18" t="str">
-        <v>2026-05-31</v>
+        <v>2026</v>
       </c>
       <c r="J18" t="str">
         <v>Current</v>
@@ -1010,10 +1010,10 @@
         <v>972.75</v>
       </c>
       <c r="H19" t="str">
-        <v>2025-06-01</v>
+        <v>2025</v>
       </c>
       <c r="I19" t="str">
-        <v>2026-06-31</v>
+        <v>2026</v>
       </c>
       <c r="J19" t="str">
         <v>Current</v>
@@ -1042,10 +1042,10 @@
         <v>1034.25</v>
       </c>
       <c r="H20" t="str">
-        <v>2025-08-01</v>
+        <v>2025</v>
       </c>
       <c r="I20" t="str">
-        <v>2026-08-31</v>
+        <v>2026</v>
       </c>
       <c r="J20" t="str">
         <v>Current</v>
@@ -1074,10 +1074,10 @@
         <v>962.25</v>
       </c>
       <c r="H21" t="str">
-        <v>2025-06-01</v>
+        <v>2025</v>
       </c>
       <c r="I21" t="str">
-        <v>2026-06-31</v>
+        <v>2026</v>
       </c>
       <c r="J21" t="str">
         <v>Current</v>
@@ -1106,10 +1106,10 @@
         <v>993</v>
       </c>
       <c r="H22" t="str">
-        <v>2025-07-01</v>
+        <v>2025</v>
       </c>
       <c r="I22" t="str">
-        <v>2026-07-31</v>
+        <v>2026</v>
       </c>
       <c r="J22" t="str">
         <v>Current</v>
@@ -1138,10 +1138,10 @@
         <v>1023.75</v>
       </c>
       <c r="H23" t="str">
-        <v>2025-08-01</v>
+        <v>2025</v>
       </c>
       <c r="I23" t="str">
-        <v>2026-08-31</v>
+        <v>2026</v>
       </c>
       <c r="J23" t="str">
         <v>Current</v>
@@ -1170,10 +1170,10 @@
         <v>1054.5</v>
       </c>
       <c r="H24" t="str">
-        <v>2025-09-01</v>
+        <v>2025</v>
       </c>
       <c r="I24" t="str">
-        <v>2026-09-31</v>
+        <v>2026</v>
       </c>
       <c r="J24" t="str">
         <v>Current</v>
@@ -1202,10 +1202,10 @@
         <v>962.25</v>
       </c>
       <c r="H25" t="str">
-        <v>2025-06-01</v>
+        <v>2025</v>
       </c>
       <c r="I25" t="str">
-        <v>2026-06-31</v>
+        <v>2026</v>
       </c>
       <c r="J25" t="str">
         <v>Current</v>
@@ -1234,10 +1234,10 @@
         <v>993</v>
       </c>
       <c r="H26" t="str">
-        <v>2025-07-01</v>
+        <v>2025</v>
       </c>
       <c r="I26" t="str">
-        <v>2026-07-31</v>
+        <v>2026</v>
       </c>
       <c r="J26" t="str">
         <v>Current</v>
@@ -1266,10 +1266,10 @@
         <v>1054.5</v>
       </c>
       <c r="H27" t="str">
-        <v>2025-09-01</v>
+        <v>2025</v>
       </c>
       <c r="I27" t="str">
-        <v>2026-09-31</v>
+        <v>2026</v>
       </c>
       <c r="J27" t="str">
         <v>Current</v>
@@ -1298,10 +1298,10 @@
         <v>1085.25</v>
       </c>
       <c r="H28" t="str">
-        <v>2025-10-01</v>
+        <v>2025</v>
       </c>
       <c r="I28" t="str">
-        <v>2026-10-31</v>
+        <v>2026</v>
       </c>
       <c r="J28" t="str">
         <v>Current</v>
@@ -1330,10 +1330,10 @@
         <v>962.25</v>
       </c>
       <c r="H29" t="str">
-        <v>2025-06-01</v>
+        <v>2025</v>
       </c>
       <c r="I29" t="str">
-        <v>2026-06-31</v>
+        <v>2026</v>
       </c>
       <c r="J29" t="str">
         <v>Current</v>
@@ -1362,10 +1362,10 @@
         <v>993</v>
       </c>
       <c r="H30" t="str">
-        <v>2025-07-01</v>
+        <v>2025</v>
       </c>
       <c r="I30" t="str">
-        <v>2026-07-31</v>
+        <v>2026</v>
       </c>
       <c r="J30" t="str">
         <v>Current</v>
@@ -1394,10 +1394,10 @@
         <v>1023.75</v>
       </c>
       <c r="H31" t="str">
-        <v>2025-08-01</v>
+        <v>2025</v>
       </c>
       <c r="I31" t="str">
-        <v>2026-08-31</v>
+        <v>2026</v>
       </c>
       <c r="J31" t="str">
         <v>Current</v>
@@ -1426,10 +1426,10 @@
         <v>962.25</v>
       </c>
       <c r="H32" t="str">
-        <v>2025-06-01</v>
+        <v>2025</v>
       </c>
       <c r="I32" t="str">
-        <v>2026-06-31</v>
+        <v>2026</v>
       </c>
       <c r="J32" t="str">
         <v>Current</v>
@@ -1458,10 +1458,10 @@
         <v>993</v>
       </c>
       <c r="H33" t="str">
-        <v>2025-07-01</v>
+        <v>2025</v>
       </c>
       <c r="I33" t="str">
-        <v>2026-07-31</v>
+        <v>2026</v>
       </c>
       <c r="J33" t="str">
         <v>Notice</v>
@@ -1490,10 +1490,10 @@
         <v>1023.75</v>
       </c>
       <c r="H34" t="str">
-        <v>2025-08-01</v>
+        <v>2025</v>
       </c>
       <c r="I34" t="str">
-        <v>2026-08-31</v>
+        <v>2026</v>
       </c>
       <c r="J34" t="str">
         <v>Current</v>
@@ -1522,10 +1522,10 @@
         <v>962.25</v>
       </c>
       <c r="H35" t="str">
-        <v>2025-06-01</v>
+        <v>2025</v>
       </c>
       <c r="I35" t="str">
-        <v>2026-06-31</v>
+        <v>2026</v>
       </c>
       <c r="J35" t="str">
         <v>Current</v>
@@ -1554,10 +1554,10 @@
         <v>993</v>
       </c>
       <c r="H36" t="str">
-        <v>2025-07-01</v>
+        <v>2025</v>
       </c>
       <c r="I36" t="str">
-        <v>2026-07-31</v>
+        <v>2026</v>
       </c>
       <c r="J36" t="str">
         <v>Current</v>
@@ -1586,10 +1586,10 @@
         <v>1054.5</v>
       </c>
       <c r="H37" t="str">
-        <v>2025-09-01</v>
+        <v>2025</v>
       </c>
       <c r="I37" t="str">
-        <v>2026-09-31</v>
+        <v>2026</v>
       </c>
       <c r="J37" t="str">
         <v>Current</v>
@@ -1618,10 +1618,10 @@
         <v>1085.25</v>
       </c>
       <c r="H38" t="str">
-        <v>2025-10-01</v>
+        <v>2025</v>
       </c>
       <c r="I38" t="str">
-        <v>2026-10-31</v>
+        <v>2026</v>
       </c>
       <c r="J38" t="str">
         <v>Current</v>
@@ -1650,10 +1650,10 @@
         <v>962.25</v>
       </c>
       <c r="H39" t="str">
-        <v>2025-06-01</v>
+        <v>2025</v>
       </c>
       <c r="I39" t="str">
-        <v>2026-06-31</v>
+        <v>2026</v>
       </c>
       <c r="J39" t="str">
         <v>Future</v>
@@ -1682,10 +1682,10 @@
         <v>993</v>
       </c>
       <c r="H40" t="str">
-        <v>2025-07-01</v>
+        <v>2025</v>
       </c>
       <c r="I40" t="str">
-        <v>2026-07-31</v>
+        <v>2026</v>
       </c>
       <c r="J40" t="str">
         <v>Future</v>
@@ -1714,10 +1714,10 @@
         <v>1023.75</v>
       </c>
       <c r="H41" t="str">
-        <v>2025-08-01</v>
+        <v>2025</v>
       </c>
       <c r="I41" t="str">
-        <v>2026-08-31</v>
+        <v>2026</v>
       </c>
       <c r="J41" t="str">
         <v>Future</v>
@@ -1746,10 +1746,10 @@
         <v>1054.5</v>
       </c>
       <c r="H42" t="str">
-        <v>2025-09-01</v>
+        <v>2025</v>
       </c>
       <c r="I42" t="str">
-        <v>2026-09-31</v>
+        <v>2026</v>
       </c>
       <c r="J42" t="str">
         <v>Future</v>
@@ -1778,10 +1778,10 @@
         <v>982.5</v>
       </c>
       <c r="H43" t="str">
-        <v>2025-07-01</v>
+        <v>2025</v>
       </c>
       <c r="I43" t="str">
-        <v>2026-07-31</v>
+        <v>2026</v>
       </c>
       <c r="J43" t="str">
         <v>Current</v>
@@ -1810,10 +1810,10 @@
         <v>1013.25</v>
       </c>
       <c r="H44" t="str">
-        <v>2025-08-01</v>
+        <v>2025</v>
       </c>
       <c r="I44" t="str">
-        <v>2026-08-31</v>
+        <v>2026</v>
       </c>
       <c r="J44" t="str">
         <v>Current</v>
@@ -1842,10 +1842,10 @@
         <v>1074.75</v>
       </c>
       <c r="H45" t="str">
-        <v>2025-10-01</v>
+        <v>2025</v>
       </c>
       <c r="I45" t="str">
-        <v>2026-10-31</v>
+        <v>2026</v>
       </c>
       <c r="J45" t="str">
         <v>Current</v>
@@ -1874,10 +1874,10 @@
         <v>982.5</v>
       </c>
       <c r="H46" t="str">
-        <v>2025-07-01</v>
+        <v>2025</v>
       </c>
       <c r="I46" t="str">
-        <v>2026-07-31</v>
+        <v>2026</v>
       </c>
       <c r="J46" t="str">
         <v>Current</v>
@@ -1906,10 +1906,10 @@
         <v>1013.25</v>
       </c>
       <c r="H47" t="str">
-        <v>2025-08-01</v>
+        <v>2025</v>
       </c>
       <c r="I47" t="str">
-        <v>2026-08-31</v>
+        <v>2026</v>
       </c>
       <c r="J47" t="str">
         <v>Current</v>
@@ -1938,10 +1938,10 @@
         <v>1044</v>
       </c>
       <c r="H48" t="str">
-        <v>2025-09-01</v>
+        <v>2025</v>
       </c>
       <c r="I48" t="str">
-        <v>2026-09-31</v>
+        <v>2026</v>
       </c>
       <c r="J48" t="str">
         <v>Current</v>
@@ -1970,10 +1970,10 @@
         <v>1074.75</v>
       </c>
       <c r="H49" t="str">
-        <v>2025-10-01</v>
+        <v>2025</v>
       </c>
       <c r="I49" t="str">
-        <v>2026-10-31</v>
+        <v>2026</v>
       </c>
       <c r="J49" t="str">
         <v>Current</v>
@@ -2002,10 +2002,10 @@
         <v>1105.5</v>
       </c>
       <c r="H50" t="str">
-        <v>2025-11-01</v>
+        <v>2025</v>
       </c>
       <c r="I50" t="str">
-        <v>2026-11-31</v>
+        <v>2026</v>
       </c>
       <c r="J50" t="str">
         <v>Current</v>
@@ -2034,10 +2034,10 @@
         <v>982.5</v>
       </c>
       <c r="H51" t="str">
-        <v>2025-07-01</v>
+        <v>2025</v>
       </c>
       <c r="I51" t="str">
-        <v>2026-07-31</v>
+        <v>2026</v>
       </c>
       <c r="J51" t="str">
         <v>Current</v>
@@ -2066,10 +2066,10 @@
         <v>1013.25</v>
       </c>
       <c r="H52" t="str">
-        <v>2025-08-01</v>
+        <v>2025</v>
       </c>
       <c r="I52" t="str">
-        <v>2026-08-31</v>
+        <v>2026</v>
       </c>
       <c r="J52" t="str">
         <v>Current</v>
@@ -2098,10 +2098,10 @@
         <v>982.5</v>
       </c>
       <c r="H53" t="str">
-        <v>2025-07-01</v>
+        <v>2025</v>
       </c>
       <c r="I53" t="str">
-        <v>2026-07-31</v>
+        <v>2026</v>
       </c>
       <c r="J53" t="str">
         <v>Current</v>
@@ -2130,10 +2130,10 @@
         <v>1013.25</v>
       </c>
       <c r="H54" t="str">
-        <v>2025-08-01</v>
+        <v>2025</v>
       </c>
       <c r="I54" t="str">
-        <v>2026-08-31</v>
+        <v>2026</v>
       </c>
       <c r="J54" t="str">
         <v>Current</v>
@@ -2162,10 +2162,10 @@
         <v>1044</v>
       </c>
       <c r="H55" t="str">
-        <v>2025-09-01</v>
+        <v>2025</v>
       </c>
       <c r="I55" t="str">
-        <v>2026-09-31</v>
+        <v>2026</v>
       </c>
       <c r="J55" t="str">
         <v>Current</v>
@@ -2194,10 +2194,10 @@
         <v>1074.75</v>
       </c>
       <c r="H56" t="str">
-        <v>2025-10-01</v>
+        <v>2025</v>
       </c>
       <c r="I56" t="str">
-        <v>2026-10-31</v>
+        <v>2026</v>
       </c>
       <c r="J56" t="str">
         <v>Current</v>
@@ -2226,10 +2226,10 @@
         <v>1105.5</v>
       </c>
       <c r="H57" t="str">
-        <v>2025-11-01</v>
+        <v>2025</v>
       </c>
       <c r="I57" t="str">
-        <v>2026-11-31</v>
+        <v>2026</v>
       </c>
       <c r="J57" t="str">
         <v>Current</v>
@@ -2258,10 +2258,10 @@
         <v>982.5</v>
       </c>
       <c r="H58" t="str">
-        <v>2025-07-01</v>
+        <v>2025</v>
       </c>
       <c r="I58" t="str">
-        <v>2026-07-31</v>
+        <v>2026</v>
       </c>
       <c r="J58" t="str">
         <v>Current</v>
@@ -2290,10 +2290,10 @@
         <v>1013.25</v>
       </c>
       <c r="H59" t="str">
-        <v>2025-08-01</v>
+        <v>2025</v>
       </c>
       <c r="I59" t="str">
-        <v>2026-08-31</v>
+        <v>2026</v>
       </c>
       <c r="J59" t="str">
         <v>Current</v>
@@ -2322,10 +2322,10 @@
         <v>1044</v>
       </c>
       <c r="H60" t="str">
-        <v>2025-09-01</v>
+        <v>2025</v>
       </c>
       <c r="I60" t="str">
-        <v>2026-09-31</v>
+        <v>2026</v>
       </c>
       <c r="J60" t="str">
         <v>Current</v>
@@ -2354,10 +2354,10 @@
         <v>1074.75</v>
       </c>
       <c r="H61" t="str">
-        <v>2025-10-01</v>
+        <v>2025</v>
       </c>
       <c r="I61" t="str">
-        <v>2026-10-31</v>
+        <v>2026</v>
       </c>
       <c r="J61" t="str">
         <v>Current</v>
@@ -2386,10 +2386,10 @@
         <v>1002.75</v>
       </c>
       <c r="H62" t="str">
-        <v>2025-08-01</v>
+        <v>2025</v>
       </c>
       <c r="I62" t="str">
-        <v>2026-08-31</v>
+        <v>2026</v>
       </c>
       <c r="J62" t="str">
         <v>Current</v>
@@ -2418,10 +2418,10 @@
         <v>1033.5</v>
       </c>
       <c r="H63" t="str">
-        <v>2025-09-01</v>
+        <v>2025</v>
       </c>
       <c r="I63" t="str">
-        <v>2026-09-31</v>
+        <v>2026</v>
       </c>
       <c r="J63" t="str">
         <v>Current</v>
@@ -2450,10 +2450,10 @@
         <v>1064.25</v>
       </c>
       <c r="H64" t="str">
-        <v>2025-10-01</v>
+        <v>2025</v>
       </c>
       <c r="I64" t="str">
-        <v>2026-10-31</v>
+        <v>2026</v>
       </c>
       <c r="J64" t="str">
         <v>Current</v>
@@ -2482,10 +2482,10 @@
         <v>1095</v>
       </c>
       <c r="H65" t="str">
-        <v>2025-11-01</v>
+        <v>2025</v>
       </c>
       <c r="I65" t="str">
-        <v>2026-11-31</v>
+        <v>2026</v>
       </c>
       <c r="J65" t="str">
         <v>Current</v>
@@ -2514,10 +2514,10 @@
         <v>1002.75</v>
       </c>
       <c r="H66" t="str">
-        <v>2025-08-01</v>
+        <v>2025</v>
       </c>
       <c r="I66" t="str">
-        <v>2026-08-31</v>
+        <v>2026</v>
       </c>
       <c r="J66" t="str">
         <v>Current</v>
@@ -2546,10 +2546,10 @@
         <v>1033.5</v>
       </c>
       <c r="H67" t="str">
-        <v>2025-09-01</v>
+        <v>2025</v>
       </c>
       <c r="I67" t="str">
-        <v>2026-09-31</v>
+        <v>2026</v>
       </c>
       <c r="J67" t="str">
         <v>Notice</v>
@@ -2578,10 +2578,10 @@
         <v>1064.25</v>
       </c>
       <c r="H68" t="str">
-        <v>2025-10-01</v>
+        <v>2025</v>
       </c>
       <c r="I68" t="str">
-        <v>2026-10-31</v>
+        <v>2026</v>
       </c>
       <c r="J68" t="str">
         <v>Current</v>
@@ -2610,10 +2610,10 @@
         <v>1095</v>
       </c>
       <c r="H69" t="str">
-        <v>2025-11-01</v>
+        <v>2025</v>
       </c>
       <c r="I69" t="str">
-        <v>2026-11-31</v>
+        <v>2026</v>
       </c>
       <c r="J69" t="str">
         <v>Current</v>
@@ -2642,10 +2642,10 @@
         <v>1125.75</v>
       </c>
       <c r="H70" t="str">
-        <v>2025-12-01</v>
+        <v>2025</v>
       </c>
       <c r="I70" t="str">
-        <v>2026-12-31</v>
+        <v>2026</v>
       </c>
       <c r="J70" t="str">
         <v>Current</v>
@@ -2674,10 +2674,10 @@
         <v>1002.75</v>
       </c>
       <c r="H71" t="str">
-        <v>2025-08-01</v>
+        <v>2025</v>
       </c>
       <c r="I71" t="str">
-        <v>2026-08-31</v>
+        <v>2026</v>
       </c>
       <c r="J71" t="str">
         <v>Current</v>
@@ -2706,10 +2706,10 @@
         <v>1033.5</v>
       </c>
       <c r="H72" t="str">
-        <v>2025-09-01</v>
+        <v>2025</v>
       </c>
       <c r="I72" t="str">
-        <v>2026-09-31</v>
+        <v>2026</v>
       </c>
       <c r="J72" t="str">
         <v>Current</v>
@@ -2738,10 +2738,10 @@
         <v>1002.75</v>
       </c>
       <c r="H73" t="str">
-        <v>2025-08-01</v>
+        <v>2025</v>
       </c>
       <c r="I73" t="str">
-        <v>2026-08-31</v>
+        <v>2026</v>
       </c>
       <c r="J73" t="str">
         <v>Current</v>
@@ -2770,10 +2770,10 @@
         <v>1033.5</v>
       </c>
       <c r="H74" t="str">
-        <v>2025-09-01</v>
+        <v>2025</v>
       </c>
       <c r="I74" t="str">
-        <v>2026-09-31</v>
+        <v>2026</v>
       </c>
       <c r="J74" t="str">
         <v>Current</v>
@@ -2802,10 +2802,10 @@
         <v>1064.25</v>
       </c>
       <c r="H75" t="str">
-        <v>2025-10-01</v>
+        <v>2025</v>
       </c>
       <c r="I75" t="str">
-        <v>2026-10-31</v>
+        <v>2026</v>
       </c>
       <c r="J75" t="str">
         <v>Current</v>
@@ -2834,10 +2834,10 @@
         <v>1002.75</v>
       </c>
       <c r="H76" t="str">
-        <v>2025-08-01</v>
+        <v>2025</v>
       </c>
       <c r="I76" t="str">
-        <v>2026-08-31</v>
+        <v>2026</v>
       </c>
       <c r="J76" t="str">
         <v>Current</v>
@@ -2866,10 +2866,10 @@
         <v>1033.5</v>
       </c>
       <c r="H77" t="str">
-        <v>2025-09-01</v>
+        <v>2025</v>
       </c>
       <c r="I77" t="str">
-        <v>2026-09-31</v>
+        <v>2026</v>
       </c>
       <c r="J77" t="str">
         <v>Current</v>
@@ -2898,10 +2898,10 @@
         <v>1064.25</v>
       </c>
       <c r="H78" t="str">
-        <v>2025-10-01</v>
+        <v>2025</v>
       </c>
       <c r="I78" t="str">
-        <v>2026-10-31</v>
+        <v>2026</v>
       </c>
       <c r="J78" t="str">
         <v>Current</v>
@@ -2930,10 +2930,10 @@
         <v>1095</v>
       </c>
       <c r="H79" t="str">
-        <v>2025-11-01</v>
+        <v>2025</v>
       </c>
       <c r="I79" t="str">
-        <v>2026-11-31</v>
+        <v>2026</v>
       </c>
       <c r="J79" t="str">
         <v>Current</v>
@@ -2962,10 +2962,10 @@
         <v>1125.75</v>
       </c>
       <c r="H80" t="str">
-        <v>2025-12-01</v>
+        <v>2025</v>
       </c>
       <c r="I80" t="str">
-        <v>2026-12-31</v>
+        <v>2026</v>
       </c>
       <c r="J80" t="str">
         <v>Current</v>
@@ -2994,10 +2994,10 @@
         <v>1002.75</v>
       </c>
       <c r="H81" t="str">
-        <v>2025-08-01</v>
+        <v>2025</v>
       </c>
       <c r="I81" t="str">
-        <v>2026-08-31</v>
+        <v>2026</v>
       </c>
       <c r="J81" t="str">
         <v>Current</v>
@@ -3026,10 +3026,10 @@
         <v>1033.5</v>
       </c>
       <c r="H82" t="str">
-        <v>2025-09-01</v>
+        <v>2025</v>
       </c>
       <c r="I82" t="str">
-        <v>2026-09-31</v>
+        <v>2026</v>
       </c>
       <c r="J82" t="str">
         <v>Notice</v>
@@ -3058,10 +3058,10 @@
         <v>1095</v>
       </c>
       <c r="H83" t="str">
-        <v>2025-11-01</v>
+        <v>2025</v>
       </c>
       <c r="I83" t="str">
-        <v>2026-11-31</v>
+        <v>2026</v>
       </c>
       <c r="J83" t="str">
         <v>Current</v>
@@ -3090,10 +3090,10 @@
         <v>1023</v>
       </c>
       <c r="H84" t="str">
-        <v>2025-09-01</v>
+        <v>2025</v>
       </c>
       <c r="I84" t="str">
-        <v>2026-09-31</v>
+        <v>2026</v>
       </c>
       <c r="J84" t="str">
         <v>Current</v>
@@ -3122,10 +3122,10 @@
         <v>1053.75</v>
       </c>
       <c r="H85" t="str">
-        <v>2025-10-01</v>
+        <v>2025</v>
       </c>
       <c r="I85" t="str">
-        <v>2026-10-31</v>
+        <v>2026</v>
       </c>
       <c r="J85" t="str">
         <v>Notice</v>
@@ -3154,10 +3154,10 @@
         <v>1084.5</v>
       </c>
       <c r="H86" t="str">
-        <v>2025-11-01</v>
+        <v>2025</v>
       </c>
       <c r="I86" t="str">
-        <v>2026-11-31</v>
+        <v>2026</v>
       </c>
       <c r="J86" t="str">
         <v>Current</v>
@@ -3186,10 +3186,10 @@
         <v>1115.25</v>
       </c>
       <c r="H87" t="str">
-        <v>2025-12-01</v>
+        <v>2025</v>
       </c>
       <c r="I87" t="str">
-        <v>2026-12-31</v>
+        <v>2026</v>
       </c>
       <c r="J87" t="str">
         <v>Current</v>
@@ -3218,10 +3218,10 @@
         <v>1023</v>
       </c>
       <c r="H88" t="str">
-        <v>2025-09-01</v>
+        <v>2025</v>
       </c>
       <c r="I88" t="str">
-        <v>2026-09-31</v>
+        <v>2026</v>
       </c>
       <c r="J88" t="str">
         <v>Current</v>
@@ -3250,10 +3250,10 @@
         <v>1053.75</v>
       </c>
       <c r="H89" t="str">
-        <v>2025-10-01</v>
+        <v>2025</v>
       </c>
       <c r="I89" t="str">
-        <v>2026-10-31</v>
+        <v>2026</v>
       </c>
       <c r="J89" t="str">
         <v>Current</v>
@@ -3282,10 +3282,10 @@
         <v>1115.25</v>
       </c>
       <c r="H90" t="str">
-        <v>2025-12-01</v>
+        <v>2025</v>
       </c>
       <c r="I90" t="str">
-        <v>2026-12-31</v>
+        <v>2026</v>
       </c>
       <c r="J90" t="str">
         <v>Current</v>
@@ -3314,10 +3314,10 @@
         <v>1146</v>
       </c>
       <c r="H91" t="str">
-        <v>2025-01-01</v>
+        <v>2025</v>
       </c>
       <c r="I91" t="str">
-        <v>2026-01-31</v>
+        <v>2026</v>
       </c>
       <c r="J91" t="str">
         <v>Current</v>
@@ -3346,10 +3346,10 @@
         <v>1023</v>
       </c>
       <c r="H92" t="str">
-        <v>2025-09-01</v>
+        <v>2025</v>
       </c>
       <c r="I92" t="str">
-        <v>2026-09-31</v>
+        <v>2026</v>
       </c>
       <c r="J92" t="str">
         <v>Current</v>
@@ -3378,10 +3378,10 @@
         <v>1053.75</v>
       </c>
       <c r="H93" t="str">
-        <v>2025-10-01</v>
+        <v>2025</v>
       </c>
       <c r="I93" t="str">
-        <v>2026-10-31</v>
+        <v>2026</v>
       </c>
       <c r="J93" t="str">
         <v>Current</v>
@@ -3410,10 +3410,10 @@
         <v>1084.5</v>
       </c>
       <c r="H94" t="str">
-        <v>2025-11-01</v>
+        <v>2025</v>
       </c>
       <c r="I94" t="str">
-        <v>2026-11-31</v>
+        <v>2026</v>
       </c>
       <c r="J94" t="str">
         <v>Current</v>
@@ -3442,10 +3442,10 @@
         <v>1023</v>
       </c>
       <c r="H95" t="str">
-        <v>2025-09-01</v>
+        <v>2025</v>
       </c>
       <c r="I95" t="str">
-        <v>2026-09-31</v>
+        <v>2026</v>
       </c>
       <c r="J95" t="str">
         <v>Current</v>
@@ -3474,10 +3474,10 @@
         <v>1053.75</v>
       </c>
       <c r="H96" t="str">
-        <v>2025-10-01</v>
+        <v>2025</v>
       </c>
       <c r="I96" t="str">
-        <v>2026-10-31</v>
+        <v>2026</v>
       </c>
       <c r="J96" t="str">
         <v>Current</v>
@@ -3506,10 +3506,10 @@
         <v>1084.5</v>
       </c>
       <c r="H97" t="str">
-        <v>2025-11-01</v>
+        <v>2025</v>
       </c>
       <c r="I97" t="str">
-        <v>2026-11-31</v>
+        <v>2026</v>
       </c>
       <c r="J97" t="str">
         <v>Current</v>
@@ -3538,10 +3538,10 @@
         <v>1023</v>
       </c>
       <c r="H98" t="str">
-        <v>2025-09-01</v>
+        <v>2025</v>
       </c>
       <c r="I98" t="str">
-        <v>2026-09-31</v>
+        <v>2026</v>
       </c>
       <c r="J98" t="str">
         <v>Current</v>
@@ -3570,10 +3570,10 @@
         <v>1053.75</v>
       </c>
       <c r="H99" t="str">
-        <v>2025-10-01</v>
+        <v>2025</v>
       </c>
       <c r="I99" t="str">
-        <v>2026-10-31</v>
+        <v>2026</v>
       </c>
       <c r="J99" t="str">
         <v>Notice</v>
@@ -3602,10 +3602,10 @@
         <v>1115.25</v>
       </c>
       <c r="H100" t="str">
-        <v>2025-12-01</v>
+        <v>2025</v>
       </c>
       <c r="I100" t="str">
-        <v>2026-12-31</v>
+        <v>2026</v>
       </c>
       <c r="J100" t="str">
         <v>Current</v>
@@ -3634,10 +3634,10 @@
         <v>1146</v>
       </c>
       <c r="H101" t="str">
-        <v>2025-01-01</v>
+        <v>2025</v>
       </c>
       <c r="I101" t="str">
-        <v>2026-01-31</v>
+        <v>2026</v>
       </c>
       <c r="J101" t="str">
         <v>Current</v>
@@ -3666,10 +3666,10 @@
         <v>1023</v>
       </c>
       <c r="H102" t="str">
-        <v>2025-09-01</v>
+        <v>2025</v>
       </c>
       <c r="I102" t="str">
-        <v>2026-09-31</v>
+        <v>2026</v>
       </c>
       <c r="J102" t="str">
         <v>Current</v>
@@ -3698,10 +3698,10 @@
         <v>1053.75</v>
       </c>
       <c r="H103" t="str">
-        <v>2025-10-01</v>
+        <v>2025</v>
       </c>
       <c r="I103" t="str">
-        <v>2026-10-31</v>
+        <v>2026</v>
       </c>
       <c r="J103" t="str">
         <v>Current</v>
@@ -3730,10 +3730,10 @@
         <v>1084.5</v>
       </c>
       <c r="H104" t="str">
-        <v>2025-11-01</v>
+        <v>2025</v>
       </c>
       <c r="I104" t="str">
-        <v>2026-11-31</v>
+        <v>2026</v>
       </c>
       <c r="J104" t="str">
         <v>Current</v>
@@ -3762,10 +3762,10 @@
         <v>1115.25</v>
       </c>
       <c r="H105" t="str">
-        <v>2025-12-01</v>
+        <v>2025</v>
       </c>
       <c r="I105" t="str">
-        <v>2026-12-31</v>
+        <v>2026</v>
       </c>
       <c r="J105" t="str">
         <v>Current</v>
@@ -3794,10 +3794,10 @@
         <v>1043.25</v>
       </c>
       <c r="H106" t="str">
-        <v>2025-10-01</v>
+        <v>2025</v>
       </c>
       <c r="I106" t="str">
-        <v>2026-10-31</v>
+        <v>2026</v>
       </c>
       <c r="J106" t="str">
         <v>Current</v>
@@ -3826,10 +3826,10 @@
         <v>1074</v>
       </c>
       <c r="H107" t="str">
-        <v>2025-11-01</v>
+        <v>2025</v>
       </c>
       <c r="I107" t="str">
-        <v>2026-11-31</v>
+        <v>2026</v>
       </c>
       <c r="J107" t="str">
         <v>Current</v>
@@ -3858,10 +3858,10 @@
         <v>1104.75</v>
       </c>
       <c r="H108" t="str">
-        <v>2025-12-01</v>
+        <v>2025</v>
       </c>
       <c r="I108" t="str">
-        <v>2026-12-31</v>
+        <v>2026</v>
       </c>
       <c r="J108" t="str">
         <v>Current</v>
@@ -3890,10 +3890,10 @@
         <v>1135.5</v>
       </c>
       <c r="H109" t="str">
-        <v>2025-01-01</v>
+        <v>2025</v>
       </c>
       <c r="I109" t="str">
-        <v>2026-01-31</v>
+        <v>2026</v>
       </c>
       <c r="J109" t="str">
         <v>Current</v>
@@ -3922,10 +3922,10 @@
         <v>1166.25</v>
       </c>
       <c r="H110" t="str">
-        <v>2025-02-01</v>
+        <v>2025</v>
       </c>
       <c r="I110" t="str">
-        <v>2026-02-31</v>
+        <v>2026</v>
       </c>
       <c r="J110" t="str">
         <v>Current</v>
@@ -3954,10 +3954,10 @@
         <v>1043.25</v>
       </c>
       <c r="H111" t="str">
-        <v>2025-10-01</v>
+        <v>2025</v>
       </c>
       <c r="I111" t="str">
-        <v>2026-10-31</v>
+        <v>2026</v>
       </c>
       <c r="J111" t="str">
         <v>Current</v>
@@ -3986,10 +3986,10 @@
         <v>1074</v>
       </c>
       <c r="H112" t="str">
-        <v>2025-11-01</v>
+        <v>2025</v>
       </c>
       <c r="I112" t="str">
-        <v>2026-11-31</v>
+        <v>2026</v>
       </c>
       <c r="J112" t="str">
         <v>Current</v>
@@ -4018,10 +4018,10 @@
         <v>1104.75</v>
       </c>
       <c r="H113" t="str">
-        <v>2025-12-01</v>
+        <v>2025</v>
       </c>
       <c r="I113" t="str">
-        <v>2026-12-31</v>
+        <v>2026</v>
       </c>
       <c r="J113" t="str">
         <v>Current</v>
@@ -4050,10 +4050,10 @@
         <v>1043.25</v>
       </c>
       <c r="H114" t="str">
-        <v>2025-10-01</v>
+        <v>2025</v>
       </c>
       <c r="I114" t="str">
-        <v>2026-10-31</v>
+        <v>2026</v>
       </c>
       <c r="J114" t="str">
         <v>Current</v>
@@ -4082,10 +4082,10 @@
         <v>1074</v>
       </c>
       <c r="H115" t="str">
-        <v>2025-11-01</v>
+        <v>2025</v>
       </c>
       <c r="I115" t="str">
-        <v>2026-11-31</v>
+        <v>2026</v>
       </c>
       <c r="J115" t="str">
         <v>Notice</v>
@@ -4114,10 +4114,10 @@
         <v>1043.25</v>
       </c>
       <c r="H116" t="str">
-        <v>2025-10-01</v>
+        <v>2025</v>
       </c>
       <c r="I116" t="str">
-        <v>2026-10-31</v>
+        <v>2026</v>
       </c>
       <c r="J116" t="str">
         <v>Current</v>
@@ -4146,10 +4146,10 @@
         <v>1074</v>
       </c>
       <c r="H117" t="str">
-        <v>2025-11-01</v>
+        <v>2025</v>
       </c>
       <c r="I117" t="str">
-        <v>2026-11-31</v>
+        <v>2026</v>
       </c>
       <c r="J117" t="str">
         <v>Current</v>
@@ -4178,10 +4178,10 @@
         <v>1104.75</v>
       </c>
       <c r="H118" t="str">
-        <v>2025-12-01</v>
+        <v>2025</v>
       </c>
       <c r="I118" t="str">
-        <v>2026-12-31</v>
+        <v>2026</v>
       </c>
       <c r="J118" t="str">
         <v>Current</v>
@@ -4210,10 +4210,10 @@
         <v>1135.5</v>
       </c>
       <c r="H119" t="str">
-        <v>2025-01-01</v>
+        <v>2025</v>
       </c>
       <c r="I119" t="str">
-        <v>2026-01-31</v>
+        <v>2026</v>
       </c>
       <c r="J119" t="str">
         <v>Current</v>
@@ -4242,10 +4242,10 @@
         <v>1166.25</v>
       </c>
       <c r="H120" t="str">
-        <v>2025-02-01</v>
+        <v>2025</v>
       </c>
       <c r="I120" t="str">
-        <v>2026-02-31</v>
+        <v>2026</v>
       </c>
       <c r="J120" t="str">
         <v>Current</v>
@@ -4274,10 +4274,10 @@
         <v>1043.25</v>
       </c>
       <c r="H121" t="str">
-        <v>2025-10-01</v>
+        <v>2025</v>
       </c>
       <c r="I121" t="str">
-        <v>2026-10-31</v>
+        <v>2026</v>
       </c>
       <c r="J121" t="str">
         <v>Current</v>
@@ -4306,10 +4306,10 @@
         <v>1074</v>
       </c>
       <c r="H122" t="str">
-        <v>2025-11-01</v>
+        <v>2025</v>
       </c>
       <c r="I122" t="str">
-        <v>2026-11-31</v>
+        <v>2026</v>
       </c>
       <c r="J122" t="str">
         <v>Current</v>
@@ -4338,10 +4338,10 @@
         <v>1104.75</v>
       </c>
       <c r="H123" t="str">
-        <v>2025-12-01</v>
+        <v>2025</v>
       </c>
       <c r="I123" t="str">
-        <v>2026-12-31</v>
+        <v>2026</v>
       </c>
       <c r="J123" t="str">
         <v>Current</v>
@@ -4370,10 +4370,10 @@
         <v>1135.5</v>
       </c>
       <c r="H124" t="str">
-        <v>2025-01-01</v>
+        <v>2025</v>
       </c>
       <c r="I124" t="str">
-        <v>2026-01-31</v>
+        <v>2026</v>
       </c>
       <c r="J124" t="str">
         <v>Current</v>
@@ -4402,10 +4402,10 @@
         <v>1063.5</v>
       </c>
       <c r="H125" t="str">
-        <v>2025-11-01</v>
+        <v>2025</v>
       </c>
       <c r="I125" t="str">
-        <v>2026-11-31</v>
+        <v>2026</v>
       </c>
       <c r="J125" t="str">
         <v>Current</v>
@@ -4434,10 +4434,10 @@
         <v>1094.25</v>
       </c>
       <c r="H126" t="str">
-        <v>2025-12-01</v>
+        <v>2025</v>
       </c>
       <c r="I126" t="str">
-        <v>2026-12-31</v>
+        <v>2026</v>
       </c>
       <c r="J126" t="str">
         <v>Current</v>
@@ -4466,10 +4466,10 @@
         <v>1125</v>
       </c>
       <c r="H127" t="str">
-        <v>2025-01-01</v>
+        <v>2025</v>
       </c>
       <c r="I127" t="str">
-        <v>2026-01-31</v>
+        <v>2026</v>
       </c>
       <c r="J127" t="str">
         <v>Current</v>
@@ -4498,10 +4498,10 @@
         <v>1155.75</v>
       </c>
       <c r="H128" t="str">
-        <v>2025-02-01</v>
+        <v>2025</v>
       </c>
       <c r="I128" t="str">
-        <v>2026-02-31</v>
+        <v>2026</v>
       </c>
       <c r="J128" t="str">
         <v>Current</v>
@@ -4530,10 +4530,10 @@
         <v>1063.5</v>
       </c>
       <c r="H129" t="str">
-        <v>2025-11-01</v>
+        <v>2025</v>
       </c>
       <c r="I129" t="str">
-        <v>2026-11-31</v>
+        <v>2026</v>
       </c>
       <c r="J129" t="str">
         <v>Future</v>
@@ -4562,10 +4562,10 @@
         <v>1094.25</v>
       </c>
       <c r="H130" t="str">
-        <v>2025-12-01</v>
+        <v>2025</v>
       </c>
       <c r="I130" t="str">
-        <v>2026-12-31</v>
+        <v>2026</v>
       </c>
       <c r="J130" t="str">
         <v>Future</v>
@@ -4594,10 +4594,10 @@
         <v>1125</v>
       </c>
       <c r="H131" t="str">
-        <v>2025-01-01</v>
+        <v>2025</v>
       </c>
       <c r="I131" t="str">
-        <v>2026-01-31</v>
+        <v>2026</v>
       </c>
       <c r="J131" t="str">
         <v>Future</v>
@@ -4626,10 +4626,10 @@
         <v>1155.75</v>
       </c>
       <c r="H132" t="str">
-        <v>2025-02-01</v>
+        <v>2025</v>
       </c>
       <c r="I132" t="str">
-        <v>2026-02-31</v>
+        <v>2026</v>
       </c>
       <c r="J132" t="str">
         <v>Future</v>
@@ -4658,10 +4658,10 @@
         <v>1186.5</v>
       </c>
       <c r="H133" t="str">
-        <v>2025-03-01</v>
+        <v>2025</v>
       </c>
       <c r="I133" t="str">
-        <v>2026-03-31</v>
+        <v>2026</v>
       </c>
       <c r="J133" t="str">
         <v>Future</v>
@@ -4690,10 +4690,10 @@
         <v>1063.5</v>
       </c>
       <c r="H134" t="str">
-        <v>2025-11-01</v>
+        <v>2025</v>
       </c>
       <c r="I134" t="str">
-        <v>2026-11-31</v>
+        <v>2026</v>
       </c>
       <c r="J134" t="str">
         <v>Current</v>
@@ -4722,10 +4722,10 @@
         <v>1094.25</v>
       </c>
       <c r="H135" t="str">
-        <v>2025-12-01</v>
+        <v>2025</v>
       </c>
       <c r="I135" t="str">
-        <v>2026-12-31</v>
+        <v>2026</v>
       </c>
       <c r="J135" t="str">
         <v>Notice</v>
@@ -4754,10 +4754,10 @@
         <v>1063.5</v>
       </c>
       <c r="H136" t="str">
-        <v>2025-11-01</v>
+        <v>2025</v>
       </c>
       <c r="I136" t="str">
-        <v>2026-11-31</v>
+        <v>2026</v>
       </c>
       <c r="J136" t="str">
         <v>Current</v>
@@ -4786,10 +4786,10 @@
         <v>1094.25</v>
       </c>
       <c r="H137" t="str">
-        <v>2025-12-01</v>
+        <v>2025</v>
       </c>
       <c r="I137" t="str">
-        <v>2026-12-31</v>
+        <v>2026</v>
       </c>
       <c r="J137" t="str">
         <v>Current</v>
@@ -4818,10 +4818,10 @@
         <v>1125</v>
       </c>
       <c r="H138" t="str">
-        <v>2025-01-01</v>
+        <v>2025</v>
       </c>
       <c r="I138" t="str">
-        <v>2026-01-31</v>
+        <v>2026</v>
       </c>
       <c r="J138" t="str">
         <v>Current</v>
@@ -4850,10 +4850,10 @@
         <v>1063.5</v>
       </c>
       <c r="H139" t="str">
-        <v>2025-11-01</v>
+        <v>2025</v>
       </c>
       <c r="I139" t="str">
-        <v>2026-11-31</v>
+        <v>2026</v>
       </c>
       <c r="J139" t="str">
         <v>Current</v>
@@ -4882,10 +4882,10 @@
         <v>1094.25</v>
       </c>
       <c r="H140" t="str">
-        <v>2025-12-01</v>
+        <v>2025</v>
       </c>
       <c r="I140" t="str">
-        <v>2026-12-31</v>
+        <v>2026</v>
       </c>
       <c r="J140" t="str">
         <v>Current</v>
@@ -4914,10 +4914,10 @@
         <v>1125</v>
       </c>
       <c r="H141" t="str">
-        <v>2025-01-01</v>
+        <v>2025</v>
       </c>
       <c r="I141" t="str">
-        <v>2026-01-31</v>
+        <v>2026</v>
       </c>
       <c r="J141" t="str">
         <v>Current</v>
@@ -4946,10 +4946,10 @@
         <v>1155.75</v>
       </c>
       <c r="H142" t="str">
-        <v>2025-02-01</v>
+        <v>2025</v>
       </c>
       <c r="I142" t="str">
-        <v>2026-02-31</v>
+        <v>2026</v>
       </c>
       <c r="J142" t="str">
         <v>Current</v>
@@ -4978,10 +4978,10 @@
         <v>1186.5</v>
       </c>
       <c r="H143" t="str">
-        <v>2025-03-01</v>
+        <v>2025</v>
       </c>
       <c r="I143" t="str">
-        <v>2026-03-31</v>
+        <v>2026</v>
       </c>
       <c r="J143" t="str">
         <v>Current</v>
@@ -5010,10 +5010,10 @@
         <v>1063.5</v>
       </c>
       <c r="H144" t="str">
-        <v>2025-11-01</v>
+        <v>2025</v>
       </c>
       <c r="I144" t="str">
-        <v>2026-11-31</v>
+        <v>2026</v>
       </c>
       <c r="J144" t="str">
         <v>Current</v>
@@ -5042,10 +5042,10 @@
         <v>1094.25</v>
       </c>
       <c r="H145" t="str">
-        <v>2025-12-01</v>
+        <v>2025</v>
       </c>
       <c r="I145" t="str">
-        <v>2026-12-31</v>
+        <v>2026</v>
       </c>
       <c r="J145" t="str">
         <v>Current</v>
@@ -5074,10 +5074,10 @@
         <v>1155.75</v>
       </c>
       <c r="H146" t="str">
-        <v>2025-02-01</v>
+        <v>2025</v>
       </c>
       <c r="I146" t="str">
-        <v>2026-02-31</v>
+        <v>2026</v>
       </c>
       <c r="J146" t="str">
         <v>Current</v>
@@ -5106,10 +5106,10 @@
         <v>1083.75</v>
       </c>
       <c r="H147" t="str">
-        <v>2025-12-01</v>
+        <v>2025</v>
       </c>
       <c r="I147" t="str">
-        <v>2026-12-31</v>
+        <v>2026</v>
       </c>
       <c r="J147" t="str">
         <v>Current</v>
@@ -5138,10 +5138,10 @@
         <v>1114.5</v>
       </c>
       <c r="H148" t="str">
-        <v>2025-01-01</v>
+        <v>2025</v>
       </c>
       <c r="I148" t="str">
-        <v>2026-01-31</v>
+        <v>2026</v>
       </c>
       <c r="J148" t="str">
         <v>Current</v>
@@ -5170,10 +5170,10 @@
         <v>1145.25</v>
       </c>
       <c r="H149" t="str">
-        <v>2025-02-01</v>
+        <v>2025</v>
       </c>
       <c r="I149" t="str">
-        <v>2026-02-31</v>
+        <v>2026</v>
       </c>
       <c r="J149" t="str">
         <v>Current</v>
@@ -5202,10 +5202,10 @@
         <v>1176</v>
       </c>
       <c r="H150" t="str">
-        <v>2025-03-01</v>
+        <v>2025</v>
       </c>
       <c r="I150" t="str">
-        <v>2026-03-31</v>
+        <v>2026</v>
       </c>
       <c r="J150" t="str">
         <v>Current</v>
@@ -5234,10 +5234,10 @@
         <v>1083.75</v>
       </c>
       <c r="H151" t="str">
-        <v>2025-12-01</v>
+        <v>2025</v>
       </c>
       <c r="I151" t="str">
-        <v>2026-12-31</v>
+        <v>2026</v>
       </c>
       <c r="J151" t="str">
         <v>Current</v>
@@ -5266,10 +5266,10 @@
         <v>1114.5</v>
       </c>
       <c r="H152" t="str">
-        <v>2025-01-01</v>
+        <v>2025</v>
       </c>
       <c r="I152" t="str">
-        <v>2026-01-31</v>
+        <v>2026</v>
       </c>
       <c r="J152" t="str">
         <v>Notice</v>
@@ -5298,10 +5298,10 @@
         <v>1176</v>
       </c>
       <c r="H153" t="str">
-        <v>2025-03-01</v>
+        <v>2025</v>
       </c>
       <c r="I153" t="str">
-        <v>2026-03-31</v>
+        <v>2026</v>
       </c>
       <c r="J153" t="str">
         <v>Current</v>
@@ -5330,10 +5330,10 @@
         <v>1206.75</v>
       </c>
       <c r="H154" t="str">
-        <v>2025-04-01</v>
+        <v>2025</v>
       </c>
       <c r="I154" t="str">
-        <v>2026-04-31</v>
+        <v>2026</v>
       </c>
       <c r="J154" t="str">
         <v>Current</v>
@@ -5362,10 +5362,10 @@
         <v>1083.75</v>
       </c>
       <c r="H155" t="str">
-        <v>2025-12-01</v>
+        <v>2025</v>
       </c>
       <c r="I155" t="str">
-        <v>2026-12-31</v>
+        <v>2026</v>
       </c>
       <c r="J155" t="str">
         <v>Current</v>
@@ -5394,10 +5394,10 @@
         <v>1114.5</v>
       </c>
       <c r="H156" t="str">
-        <v>2025-01-01</v>
+        <v>2025</v>
       </c>
       <c r="I156" t="str">
-        <v>2026-01-31</v>
+        <v>2026</v>
       </c>
       <c r="J156" t="str">
         <v>Current</v>
@@ -5426,10 +5426,10 @@
         <v>1145.25</v>
       </c>
       <c r="H157" t="str">
-        <v>2025-02-01</v>
+        <v>2025</v>
       </c>
       <c r="I157" t="str">
-        <v>2026-02-31</v>
+        <v>2026</v>
       </c>
       <c r="J157" t="str">
         <v>Current</v>
@@ -5458,10 +5458,10 @@
         <v>1083.75</v>
       </c>
       <c r="H158" t="str">
-        <v>2025-12-01</v>
+        <v>2025</v>
       </c>
       <c r="I158" t="str">
-        <v>2026-12-31</v>
+        <v>2026</v>
       </c>
       <c r="J158" t="str">
         <v>Current</v>
@@ -5490,10 +5490,10 @@
         <v>1114.5</v>
       </c>
       <c r="H159" t="str">
-        <v>2025-01-01</v>
+        <v>2025</v>
       </c>
       <c r="I159" t="str">
-        <v>2026-01-31</v>
+        <v>2026</v>
       </c>
       <c r="J159" t="str">
         <v>Current</v>
@@ -5522,10 +5522,10 @@
         <v>1145.25</v>
       </c>
       <c r="H160" t="str">
-        <v>2025-02-01</v>
+        <v>2025</v>
       </c>
       <c r="I160" t="str">
-        <v>2026-02-31</v>
+        <v>2026</v>
       </c>
       <c r="J160" t="str">
         <v>Current</v>
@@ -5554,10 +5554,10 @@
         <v>1083.75</v>
       </c>
       <c r="H161" t="str">
-        <v>2025-12-01</v>
+        <v>2025</v>
       </c>
       <c r="I161" t="str">
-        <v>2026-12-31</v>
+        <v>2026</v>
       </c>
       <c r="J161" t="str">
         <v>Current</v>
@@ -5586,10 +5586,10 @@
         <v>1114.5</v>
       </c>
       <c r="H162" t="str">
-        <v>2025-01-01</v>
+        <v>2025</v>
       </c>
       <c r="I162" t="str">
-        <v>2026-01-31</v>
+        <v>2026</v>
       </c>
       <c r="J162" t="str">
         <v>Current</v>
@@ -5618,10 +5618,10 @@
         <v>1176</v>
       </c>
       <c r="H163" t="str">
-        <v>2025-03-01</v>
+        <v>2025</v>
       </c>
       <c r="I163" t="str">
-        <v>2026-03-31</v>
+        <v>2026</v>
       </c>
       <c r="J163" t="str">
         <v>Current</v>
@@ -5650,10 +5650,10 @@
         <v>1206.75</v>
       </c>
       <c r="H164" t="str">
-        <v>2025-04-01</v>
+        <v>2025</v>
       </c>
       <c r="I164" t="str">
-        <v>2026-04-31</v>
+        <v>2026</v>
       </c>
       <c r="J164" t="str">
         <v>Current</v>
@@ -5682,10 +5682,10 @@
         <v>1083.75</v>
       </c>
       <c r="H165" t="str">
-        <v>2025-12-01</v>
+        <v>2025</v>
       </c>
       <c r="I165" t="str">
-        <v>2026-12-31</v>
+        <v>2026</v>
       </c>
       <c r="J165" t="str">
         <v>Current</v>
@@ -5714,10 +5714,10 @@
         <v>1114.5</v>
       </c>
       <c r="H166" t="str">
-        <v>2025-01-01</v>
+        <v>2025</v>
       </c>
       <c r="I166" t="str">
-        <v>2026-01-31</v>
+        <v>2026</v>
       </c>
       <c r="J166" t="str">
         <v>Notice</v>
@@ -5746,10 +5746,10 @@
         <v>1145.25</v>
       </c>
       <c r="H167" t="str">
-        <v>2025-02-01</v>
+        <v>2025</v>
       </c>
       <c r="I167" t="str">
-        <v>2026-02-31</v>
+        <v>2026</v>
       </c>
       <c r="J167" t="str">
         <v>Current</v>
@@ -5778,10 +5778,10 @@
         <v>1176</v>
       </c>
       <c r="H168" t="str">
-        <v>2025-03-01</v>
+        <v>2025</v>
       </c>
       <c r="I168" t="str">
-        <v>2026-03-31</v>
+        <v>2026</v>
       </c>
       <c r="J168" t="str">
         <v>Current</v>
@@ -5810,10 +5810,10 @@
         <v>1104</v>
       </c>
       <c r="H169" t="str">
-        <v>2025-01-01</v>
+        <v>2025</v>
       </c>
       <c r="I169" t="str">
-        <v>2026-01-31</v>
+        <v>2026</v>
       </c>
       <c r="J169" t="str">
         <v>Current</v>
@@ -5842,10 +5842,10 @@
         <v>1134.75</v>
       </c>
       <c r="H170" t="str">
-        <v>2025-02-01</v>
+        <v>2025</v>
       </c>
       <c r="I170" t="str">
-        <v>2026-02-31</v>
+        <v>2026</v>
       </c>
       <c r="J170" t="str">
         <v>Notice</v>
@@ -5874,10 +5874,10 @@
         <v>1196.25</v>
       </c>
       <c r="H171" t="str">
-        <v>2025-04-01</v>
+        <v>2025</v>
       </c>
       <c r="I171" t="str">
-        <v>2026-04-31</v>
+        <v>2026</v>
       </c>
       <c r="J171" t="str">
         <v>Current</v>
@@ -5906,10 +5906,10 @@
         <v>1104</v>
       </c>
       <c r="H172" t="str">
-        <v>2025-01-01</v>
+        <v>2025</v>
       </c>
       <c r="I172" t="str">
-        <v>2026-01-31</v>
+        <v>2026</v>
       </c>
       <c r="J172" t="str">
         <v>Current</v>
@@ -5938,10 +5938,10 @@
         <v>1134.75</v>
       </c>
       <c r="H173" t="str">
-        <v>2025-02-01</v>
+        <v>2025</v>
       </c>
       <c r="I173" t="str">
-        <v>2026-02-31</v>
+        <v>2026</v>
       </c>
       <c r="J173" t="str">
         <v>Current</v>
@@ -5970,10 +5970,10 @@
         <v>1165.5</v>
       </c>
       <c r="H174" t="str">
-        <v>2025-03-01</v>
+        <v>2025</v>
       </c>
       <c r="I174" t="str">
-        <v>2026-03-31</v>
+        <v>2026</v>
       </c>
       <c r="J174" t="str">
         <v>Current</v>
@@ -6002,10 +6002,10 @@
         <v>1196.25</v>
       </c>
       <c r="H175" t="str">
-        <v>2025-04-01</v>
+        <v>2025</v>
       </c>
       <c r="I175" t="str">
-        <v>2026-04-31</v>
+        <v>2026</v>
       </c>
       <c r="J175" t="str">
         <v>Current</v>
@@ -6034,10 +6034,10 @@
         <v>1227</v>
       </c>
       <c r="H176" t="str">
-        <v>2025-05-01</v>
+        <v>2025</v>
       </c>
       <c r="I176" t="str">
-        <v>2026-05-31</v>
+        <v>2026</v>
       </c>
       <c r="J176" t="str">
         <v>Current</v>
@@ -6066,10 +6066,10 @@
         <v>1104</v>
       </c>
       <c r="H177" t="str">
-        <v>2025-01-01</v>
+        <v>2025</v>
       </c>
       <c r="I177" t="str">
-        <v>2026-01-31</v>
+        <v>2026</v>
       </c>
       <c r="J177" t="str">
         <v>Current</v>
@@ -6098,10 +6098,10 @@
         <v>1134.75</v>
       </c>
       <c r="H178" t="str">
-        <v>2025-02-01</v>
+        <v>2025</v>
       </c>
       <c r="I178" t="str">
-        <v>2026-02-31</v>
+        <v>2026</v>
       </c>
       <c r="J178" t="str">
         <v>Current</v>
@@ -6130,10 +6130,10 @@
         <v>1165.5</v>
       </c>
       <c r="H179" t="str">
-        <v>2025-03-01</v>
+        <v>2025</v>
       </c>
       <c r="I179" t="str">
-        <v>2026-03-31</v>
+        <v>2026</v>
       </c>
       <c r="J179" t="str">
         <v>Current</v>
@@ -6162,10 +6162,10 @@
         <v>1104</v>
       </c>
       <c r="H180" t="str">
-        <v>2025-01-01</v>
+        <v>2025</v>
       </c>
       <c r="I180" t="str">
-        <v>2026-01-31</v>
+        <v>2026</v>
       </c>
       <c r="J180" t="str">
         <v>Current</v>
@@ -6194,10 +6194,10 @@
         <v>1134.75</v>
       </c>
       <c r="H181" t="str">
-        <v>2025-02-01</v>
+        <v>2025</v>
       </c>
       <c r="I181" t="str">
-        <v>2026-02-31</v>
+        <v>2026</v>
       </c>
       <c r="J181" t="str">
         <v>Current</v>
@@ -6226,10 +6226,10 @@
         <v>1104</v>
       </c>
       <c r="H182" t="str">
-        <v>2025-01-01</v>
+        <v>2025</v>
       </c>
       <c r="I182" t="str">
-        <v>2026-01-31</v>
+        <v>2026</v>
       </c>
       <c r="J182" t="str">
         <v>Current</v>
@@ -6258,10 +6258,10 @@
         <v>1134.75</v>
       </c>
       <c r="H183" t="str">
-        <v>2025-02-01</v>
+        <v>2025</v>
       </c>
       <c r="I183" t="str">
-        <v>2026-02-31</v>
+        <v>2026</v>
       </c>
       <c r="J183" t="str">
         <v>Notice</v>
@@ -6290,10 +6290,10 @@
         <v>1165.5</v>
       </c>
       <c r="H184" t="str">
-        <v>2025-03-01</v>
+        <v>2025</v>
       </c>
       <c r="I184" t="str">
-        <v>2026-03-31</v>
+        <v>2026</v>
       </c>
       <c r="J184" t="str">
         <v>Current</v>
@@ -6322,10 +6322,10 @@
         <v>1196.25</v>
       </c>
       <c r="H185" t="str">
-        <v>2025-04-01</v>
+        <v>2025</v>
       </c>
       <c r="I185" t="str">
-        <v>2026-04-31</v>
+        <v>2026</v>
       </c>
       <c r="J185" t="str">
         <v>Current</v>
@@ -6354,10 +6354,10 @@
         <v>1227</v>
       </c>
       <c r="H186" t="str">
-        <v>2025-05-01</v>
+        <v>2025</v>
       </c>
       <c r="I186" t="str">
-        <v>2026-05-31</v>
+        <v>2026</v>
       </c>
       <c r="J186" t="str">
         <v>Current</v>
@@ -6386,10 +6386,10 @@
         <v>1104</v>
       </c>
       <c r="H187" t="str">
-        <v>2025-01-01</v>
+        <v>2025</v>
       </c>
       <c r="I187" t="str">
-        <v>2026-01-31</v>
+        <v>2026</v>
       </c>
       <c r="J187" t="str">
         <v>Current</v>
@@ -6418,10 +6418,10 @@
         <v>1134.75</v>
       </c>
       <c r="H188" t="str">
-        <v>2025-02-01</v>
+        <v>2025</v>
       </c>
       <c r="I188" t="str">
-        <v>2026-02-31</v>
+        <v>2026</v>
       </c>
       <c r="J188" t="str">
         <v>Current</v>
@@ -6450,10 +6450,10 @@
         <v>1165.5</v>
       </c>
       <c r="H189" t="str">
-        <v>2025-03-01</v>
+        <v>2025</v>
       </c>
       <c r="I189" t="str">
-        <v>2026-03-31</v>
+        <v>2026</v>
       </c>
       <c r="J189" t="str">
         <v>Current</v>
@@ -6482,10 +6482,10 @@
         <v>1196.25</v>
       </c>
       <c r="H190" t="str">
-        <v>2025-04-01</v>
+        <v>2025</v>
       </c>
       <c r="I190" t="str">
-        <v>2026-04-31</v>
+        <v>2026</v>
       </c>
       <c r="J190" t="str">
         <v>Current</v>
@@ -6514,10 +6514,10 @@
         <v>1124.25</v>
       </c>
       <c r="H191" t="str">
-        <v>2025-02-01</v>
+        <v>2025</v>
       </c>
       <c r="I191" t="str">
-        <v>2026-02-31</v>
+        <v>2026</v>
       </c>
       <c r="J191" t="str">
         <v>Current</v>
@@ -6546,10 +6546,10 @@
         <v>1155</v>
       </c>
       <c r="H192" t="str">
-        <v>2025-03-01</v>
+        <v>2025</v>
       </c>
       <c r="I192" t="str">
-        <v>2026-03-31</v>
+        <v>2026</v>
       </c>
       <c r="J192" t="str">
         <v>Current</v>
@@ -6578,10 +6578,10 @@
         <v>1185.75</v>
       </c>
       <c r="H193" t="str">
-        <v>2025-04-01</v>
+        <v>2025</v>
       </c>
       <c r="I193" t="str">
-        <v>2026-04-31</v>
+        <v>2026</v>
       </c>
       <c r="J193" t="str">
         <v>Current</v>
@@ -6610,10 +6610,10 @@
         <v>1216.5</v>
       </c>
       <c r="H194" t="str">
-        <v>2025-05-01</v>
+        <v>2025</v>
       </c>
       <c r="I194" t="str">
-        <v>2026-05-31</v>
+        <v>2026</v>
       </c>
       <c r="J194" t="str">
         <v>Current</v>
@@ -6642,10 +6642,10 @@
         <v>1124.25</v>
       </c>
       <c r="H195" t="str">
-        <v>2025-02-01</v>
+        <v>2025</v>
       </c>
       <c r="I195" t="str">
-        <v>2026-02-31</v>
+        <v>2026</v>
       </c>
       <c r="J195" t="str">
         <v>Current</v>
@@ -6674,10 +6674,10 @@
         <v>1155</v>
       </c>
       <c r="H196" t="str">
-        <v>2025-03-01</v>
+        <v>2025</v>
       </c>
       <c r="I196" t="str">
-        <v>2026-03-31</v>
+        <v>2026</v>
       </c>
       <c r="J196" t="str">
         <v>Current</v>
@@ -6706,10 +6706,10 @@
         <v>1185.75</v>
       </c>
       <c r="H197" t="str">
-        <v>2025-04-01</v>
+        <v>2025</v>
       </c>
       <c r="I197" t="str">
-        <v>2026-04-31</v>
+        <v>2026</v>
       </c>
       <c r="J197" t="str">
         <v>Current</v>
@@ -6738,10 +6738,10 @@
         <v>1216.5</v>
       </c>
       <c r="H198" t="str">
-        <v>2025-05-01</v>
+        <v>2025</v>
       </c>
       <c r="I198" t="str">
-        <v>2026-05-31</v>
+        <v>2026</v>
       </c>
       <c r="J198" t="str">
         <v>Current</v>
@@ -6770,10 +6770,10 @@
         <v>1247.25</v>
       </c>
       <c r="H199" t="str">
-        <v>2025-06-01</v>
+        <v>2025</v>
       </c>
       <c r="I199" t="str">
-        <v>2026-06-31</v>
+        <v>2026</v>
       </c>
       <c r="J199" t="str">
         <v>Current</v>
@@ -6802,10 +6802,10 @@
         <v>1124.25</v>
       </c>
       <c r="H200" t="str">
-        <v>2025-02-01</v>
+        <v>2025</v>
       </c>
       <c r="I200" t="str">
-        <v>2026-02-31</v>
+        <v>2026</v>
       </c>
       <c r="J200" t="str">
         <v>Current</v>
@@ -6834,10 +6834,10 @@
         <v>1155</v>
       </c>
       <c r="H201" t="str">
-        <v>2025-03-01</v>
+        <v>2025</v>
       </c>
       <c r="I201" t="str">
-        <v>2026-03-31</v>
+        <v>2026</v>
       </c>
       <c r="J201" t="str">
         <v>Current</v>
@@ -6866,10 +6866,10 @@
         <v>1124.25</v>
       </c>
       <c r="H202" t="str">
-        <v>2025-02-01</v>
+        <v>2025</v>
       </c>
       <c r="I202" t="str">
-        <v>2026-02-31</v>
+        <v>2026</v>
       </c>
       <c r="J202" t="str">
         <v>Current</v>
@@ -6898,10 +6898,10 @@
         <v>1155</v>
       </c>
       <c r="H203" t="str">
-        <v>2025-03-01</v>
+        <v>2025</v>
       </c>
       <c r="I203" t="str">
-        <v>2026-03-31</v>
+        <v>2026</v>
       </c>
       <c r="J203" t="str">
         <v>Current</v>
@@ -6930,10 +6930,10 @@
         <v>1185.75</v>
       </c>
       <c r="H204" t="str">
-        <v>2025-04-01</v>
+        <v>2025</v>
       </c>
       <c r="I204" t="str">
-        <v>2026-04-31</v>
+        <v>2026</v>
       </c>
       <c r="J204" t="str">
         <v>Current</v>
@@ -6962,10 +6962,10 @@
         <v>1216.5</v>
       </c>
       <c r="H205" t="str">
-        <v>2025-05-01</v>
+        <v>2025</v>
       </c>
       <c r="I205" t="str">
-        <v>2026-05-31</v>
+        <v>2026</v>
       </c>
       <c r="J205" t="str">
         <v>Current</v>
@@ -6994,10 +6994,10 @@
         <v>1247.25</v>
       </c>
       <c r="H206" t="str">
-        <v>2025-06-01</v>
+        <v>2025</v>
       </c>
       <c r="I206" t="str">
-        <v>2026-06-31</v>
+        <v>2026</v>
       </c>
       <c r="J206" t="str">
         <v>Current</v>
@@ -7026,10 +7026,10 @@
         <v>1124.25</v>
       </c>
       <c r="H207" t="str">
-        <v>2025-02-01</v>
+        <v>2025</v>
       </c>
       <c r="I207" t="str">
-        <v>2026-02-31</v>
+        <v>2026</v>
       </c>
       <c r="J207" t="str">
         <v>Current</v>
@@ -7058,10 +7058,10 @@
         <v>1155</v>
       </c>
       <c r="H208" t="str">
-        <v>2025-03-01</v>
+        <v>2025</v>
       </c>
       <c r="I208" t="str">
-        <v>2026-03-31</v>
+        <v>2026</v>
       </c>
       <c r="J208" t="str">
         <v>Current</v>
@@ -7090,10 +7090,10 @@
         <v>1216.5</v>
       </c>
       <c r="H209" t="str">
-        <v>2025-05-01</v>
+        <v>2025</v>
       </c>
       <c r="I209" t="str">
-        <v>2026-05-31</v>
+        <v>2026</v>
       </c>
       <c r="J209" t="str">
         <v>Current</v>
@@ -7122,10 +7122,10 @@
         <v>1164.75</v>
       </c>
       <c r="H210" t="str">
-        <v>2025-04-01</v>
+        <v>2025</v>
       </c>
       <c r="I210" t="str">
-        <v>2026-04-31</v>
+        <v>2026</v>
       </c>
       <c r="J210" t="str">
         <v>Current</v>
@@ -7154,10 +7154,10 @@
         <v>1195.5</v>
       </c>
       <c r="H211" t="str">
-        <v>2025-05-01</v>
+        <v>2025</v>
       </c>
       <c r="I211" t="str">
-        <v>2026-05-31</v>
+        <v>2026</v>
       </c>
       <c r="J211" t="str">
         <v>Current</v>
@@ -7186,10 +7186,10 @@
         <v>1257</v>
       </c>
       <c r="H212" t="str">
-        <v>2025-07-01</v>
+        <v>2025</v>
       </c>
       <c r="I212" t="str">
-        <v>2026-07-31</v>
+        <v>2026</v>
       </c>
       <c r="J212" t="str">
         <v>Current</v>
@@ -7218,10 +7218,10 @@
         <v>1164.75</v>
       </c>
       <c r="H213" t="str">
-        <v>2025-04-01</v>
+        <v>2025</v>
       </c>
       <c r="I213" t="str">
-        <v>2026-04-31</v>
+        <v>2026</v>
       </c>
       <c r="J213" t="str">
         <v>Current</v>
@@ -7250,10 +7250,10 @@
         <v>1195.5</v>
       </c>
       <c r="H214" t="str">
-        <v>2025-05-01</v>
+        <v>2025</v>
       </c>
       <c r="I214" t="str">
-        <v>2026-05-31</v>
+        <v>2026</v>
       </c>
       <c r="J214" t="str">
         <v>Notice</v>
@@ -7282,10 +7282,10 @@
         <v>1226.25</v>
       </c>
       <c r="H215" t="str">
-        <v>2025-06-01</v>
+        <v>2025</v>
       </c>
       <c r="I215" t="str">
-        <v>2026-06-31</v>
+        <v>2026</v>
       </c>
       <c r="J215" t="str">
         <v>Current</v>
@@ -7314,10 +7314,10 @@
         <v>1257</v>
       </c>
       <c r="H216" t="str">
-        <v>2025-07-01</v>
+        <v>2025</v>
       </c>
       <c r="I216" t="str">
-        <v>2026-07-31</v>
+        <v>2026</v>
       </c>
       <c r="J216" t="str">
         <v>Current</v>
@@ -7346,10 +7346,10 @@
         <v>1287.75</v>
       </c>
       <c r="H217" t="str">
-        <v>2025-08-01</v>
+        <v>2025</v>
       </c>
       <c r="I217" t="str">
-        <v>2026-08-31</v>
+        <v>2026</v>
       </c>
       <c r="J217" t="str">
         <v>Current</v>
@@ -7378,10 +7378,10 @@
         <v>1164.75</v>
       </c>
       <c r="H218" t="str">
-        <v>2025-04-01</v>
+        <v>2025</v>
       </c>
       <c r="I218" t="str">
-        <v>2026-04-31</v>
+        <v>2026</v>
       </c>
       <c r="J218" t="str">
         <v>Current</v>
@@ -7410,10 +7410,10 @@
         <v>1195.5</v>
       </c>
       <c r="H219" t="str">
-        <v>2025-05-01</v>
+        <v>2025</v>
       </c>
       <c r="I219" t="str">
-        <v>2026-05-31</v>
+        <v>2026</v>
       </c>
       <c r="J219" t="str">
         <v>Current</v>
@@ -7442,10 +7442,10 @@
         <v>1226.25</v>
       </c>
       <c r="H220" t="str">
-        <v>2025-06-01</v>
+        <v>2025</v>
       </c>
       <c r="I220" t="str">
-        <v>2026-06-31</v>
+        <v>2026</v>
       </c>
       <c r="J220" t="str">
         <v>Current</v>
@@ -7474,10 +7474,10 @@
         <v>1164.75</v>
       </c>
       <c r="H221" t="str">
-        <v>2025-04-01</v>
+        <v>2025</v>
       </c>
       <c r="I221" t="str">
-        <v>2026-04-31</v>
+        <v>2026</v>
       </c>
       <c r="J221" t="str">
         <v>Current</v>
@@ -7506,10 +7506,10 @@
         <v>1195.5</v>
       </c>
       <c r="H222" t="str">
-        <v>2025-05-01</v>
+        <v>2025</v>
       </c>
       <c r="I222" t="str">
-        <v>2026-05-31</v>
+        <v>2026</v>
       </c>
       <c r="J222" t="str">
         <v>Current</v>
@@ -7538,10 +7538,10 @@
         <v>1164.75</v>
       </c>
       <c r="H223" t="str">
-        <v>2025-04-01</v>
+        <v>2025</v>
       </c>
       <c r="I223" t="str">
-        <v>2026-04-31</v>
+        <v>2026</v>
       </c>
       <c r="J223" t="str">
         <v>Future</v>
@@ -7570,10 +7570,10 @@
         <v>1195.5</v>
       </c>
       <c r="H224" t="str">
-        <v>2025-05-01</v>
+        <v>2025</v>
       </c>
       <c r="I224" t="str">
-        <v>2026-05-31</v>
+        <v>2026</v>
       </c>
       <c r="J224" t="str">
         <v>Future</v>
@@ -7602,10 +7602,10 @@
         <v>1226.25</v>
       </c>
       <c r="H225" t="str">
-        <v>2025-06-01</v>
+        <v>2025</v>
       </c>
       <c r="I225" t="str">
-        <v>2026-06-31</v>
+        <v>2026</v>
       </c>
       <c r="J225" t="str">
         <v>Future</v>
@@ -7634,10 +7634,10 @@
         <v>1257</v>
       </c>
       <c r="H226" t="str">
-        <v>2025-07-01</v>
+        <v>2025</v>
       </c>
       <c r="I226" t="str">
-        <v>2026-07-31</v>
+        <v>2026</v>
       </c>
       <c r="J226" t="str">
         <v>Future</v>
@@ -7666,10 +7666,10 @@
         <v>1287.75</v>
       </c>
       <c r="H227" t="str">
-        <v>2025-08-01</v>
+        <v>2025</v>
       </c>
       <c r="I227" t="str">
-        <v>2026-08-31</v>
+        <v>2026</v>
       </c>
       <c r="J227" t="str">
         <v>Future</v>
@@ -7698,10 +7698,10 @@
         <v>1164.75</v>
       </c>
       <c r="H228" t="str">
-        <v>2025-04-01</v>
+        <v>2025</v>
       </c>
       <c r="I228" t="str">
-        <v>2026-04-31</v>
+        <v>2026</v>
       </c>
       <c r="J228" t="str">
         <v>Current</v>
@@ -7730,10 +7730,10 @@
         <v>1195.5</v>
       </c>
       <c r="H229" t="str">
-        <v>2025-05-01</v>
+        <v>2025</v>
       </c>
       <c r="I229" t="str">
-        <v>2026-05-31</v>
+        <v>2026</v>
       </c>
       <c r="J229" t="str">
         <v>Notice</v>
@@ -7762,10 +7762,10 @@
         <v>1226.25</v>
       </c>
       <c r="H230" t="str">
-        <v>2025-06-01</v>
+        <v>2025</v>
       </c>
       <c r="I230" t="str">
-        <v>2026-06-31</v>
+        <v>2026</v>
       </c>
       <c r="J230" t="str">
         <v>Current</v>
@@ -7794,10 +7794,10 @@
         <v>1257</v>
       </c>
       <c r="H231" t="str">
-        <v>2025-07-01</v>
+        <v>2025</v>
       </c>
       <c r="I231" t="str">
-        <v>2026-07-31</v>
+        <v>2026</v>
       </c>
       <c r="J231" t="str">
         <v>Current</v>
@@ -7826,10 +7826,10 @@
         <v>1185</v>
       </c>
       <c r="H232" t="str">
-        <v>2025-05-01</v>
+        <v>2025</v>
       </c>
       <c r="I232" t="str">
-        <v>2026-05-31</v>
+        <v>2026</v>
       </c>
       <c r="J232" t="str">
         <v>Current</v>
@@ -7858,10 +7858,10 @@
         <v>1215.75</v>
       </c>
       <c r="H233" t="str">
-        <v>2025-06-01</v>
+        <v>2025</v>
       </c>
       <c r="I233" t="str">
-        <v>2026-06-31</v>
+        <v>2026</v>
       </c>
       <c r="J233" t="str">
         <v>Notice</v>
@@ -7890,10 +7890,10 @@
         <v>1246.5</v>
       </c>
       <c r="H234" t="str">
-        <v>2025-07-01</v>
+        <v>2025</v>
       </c>
       <c r="I234" t="str">
-        <v>2026-07-31</v>
+        <v>2026</v>
       </c>
       <c r="J234" t="str">
         <v>Current</v>
@@ -7922,10 +7922,10 @@
         <v>1277.25</v>
       </c>
       <c r="H235" t="str">
-        <v>2025-08-01</v>
+        <v>2025</v>
       </c>
       <c r="I235" t="str">
-        <v>2026-08-31</v>
+        <v>2026</v>
       </c>
       <c r="J235" t="str">
         <v>Current</v>
@@ -7954,10 +7954,10 @@
         <v>1185</v>
       </c>
       <c r="H236" t="str">
-        <v>2025-05-01</v>
+        <v>2025</v>
       </c>
       <c r="I236" t="str">
-        <v>2026-05-31</v>
+        <v>2026</v>
       </c>
       <c r="J236" t="str">
         <v>Current</v>
@@ -7986,10 +7986,10 @@
         <v>1215.75</v>
       </c>
       <c r="H237" t="str">
-        <v>2025-06-01</v>
+        <v>2025</v>
       </c>
       <c r="I237" t="str">
-        <v>2026-06-31</v>
+        <v>2026</v>
       </c>
       <c r="J237" t="str">
         <v>Current</v>
@@ -8018,10 +8018,10 @@
         <v>1246.5</v>
       </c>
       <c r="H238" t="str">
-        <v>2025-07-01</v>
+        <v>2025</v>
       </c>
       <c r="I238" t="str">
-        <v>2026-07-31</v>
+        <v>2026</v>
       </c>
       <c r="J238" t="str">
         <v>Current</v>
@@ -8050,10 +8050,10 @@
         <v>1277.25</v>
       </c>
       <c r="H239" t="str">
-        <v>2025-08-01</v>
+        <v>2025</v>
       </c>
       <c r="I239" t="str">
-        <v>2026-08-31</v>
+        <v>2026</v>
       </c>
       <c r="J239" t="str">
         <v>Current</v>
@@ -8082,10 +8082,10 @@
         <v>1308</v>
       </c>
       <c r="H240" t="str">
-        <v>2025-09-01</v>
+        <v>2025</v>
       </c>
       <c r="I240" t="str">
-        <v>2026-09-31</v>
+        <v>2026</v>
       </c>
       <c r="J240" t="str">
         <v>Current</v>
@@ -8114,10 +8114,10 @@
         <v>1185</v>
       </c>
       <c r="H241" t="str">
-        <v>2025-05-01</v>
+        <v>2025</v>
       </c>
       <c r="I241" t="str">
-        <v>2026-05-31</v>
+        <v>2026</v>
       </c>
       <c r="J241" t="str">
         <v>Current</v>
@@ -8146,10 +8146,10 @@
         <v>1215.75</v>
       </c>
       <c r="H242" t="str">
-        <v>2025-06-01</v>
+        <v>2025</v>
       </c>
       <c r="I242" t="str">
-        <v>2026-06-31</v>
+        <v>2026</v>
       </c>
       <c r="J242" t="str">
         <v>Current</v>
@@ -8178,10 +8178,10 @@
         <v>1185</v>
       </c>
       <c r="H243" t="str">
-        <v>2025-05-01</v>
+        <v>2025</v>
       </c>
       <c r="I243" t="str">
-        <v>2026-05-31</v>
+        <v>2026</v>
       </c>
       <c r="J243" t="str">
         <v>Current</v>
@@ -8210,10 +8210,10 @@
         <v>1215.75</v>
       </c>
       <c r="H244" t="str">
-        <v>2025-06-01</v>
+        <v>2025</v>
       </c>
       <c r="I244" t="str">
-        <v>2026-06-31</v>
+        <v>2026</v>
       </c>
       <c r="J244" t="str">
         <v>Current</v>
@@ -8242,10 +8242,10 @@
         <v>1246.5</v>
       </c>
       <c r="H245" t="str">
-        <v>2025-07-01</v>
+        <v>2025</v>
       </c>
       <c r="I245" t="str">
-        <v>2026-07-31</v>
+        <v>2026</v>
       </c>
       <c r="J245" t="str">
         <v>Current</v>
@@ -8274,10 +8274,10 @@
         <v>1185</v>
       </c>
       <c r="H246" t="str">
-        <v>2025-05-01</v>
+        <v>2025</v>
       </c>
       <c r="I246" t="str">
-        <v>2026-05-31</v>
+        <v>2026</v>
       </c>
       <c r="J246" t="str">
         <v>Current</v>
@@ -8306,10 +8306,10 @@
         <v>1215.75</v>
       </c>
       <c r="H247" t="str">
-        <v>2025-06-01</v>
+        <v>2025</v>
       </c>
       <c r="I247" t="str">
-        <v>2026-06-31</v>
+        <v>2026</v>
       </c>
       <c r="J247" t="str">
         <v>Notice</v>
@@ -8338,10 +8338,10 @@
         <v>1246.5</v>
       </c>
       <c r="H248" t="str">
-        <v>2025-07-01</v>
+        <v>2025</v>
       </c>
       <c r="I248" t="str">
-        <v>2026-07-31</v>
+        <v>2026</v>
       </c>
       <c r="J248" t="str">
         <v>Current</v>
@@ -8370,10 +8370,10 @@
         <v>1277.25</v>
       </c>
       <c r="H249" t="str">
-        <v>2025-08-01</v>
+        <v>2025</v>
       </c>
       <c r="I249" t="str">
-        <v>2026-08-31</v>
+        <v>2026</v>
       </c>
       <c r="J249" t="str">
         <v>Current</v>
@@ -8402,10 +8402,10 @@
         <v>1308</v>
       </c>
       <c r="H250" t="str">
-        <v>2025-09-01</v>
+        <v>2025</v>
       </c>
       <c r="I250" t="str">
-        <v>2026-09-31</v>
+        <v>2026</v>
       </c>
       <c r="J250" t="str">
         <v>Current</v>
@@ -8434,10 +8434,10 @@
         <v>1185</v>
       </c>
       <c r="H251" t="str">
-        <v>2025-05-01</v>
+        <v>2025</v>
       </c>
       <c r="I251" t="str">
-        <v>2026-05-31</v>
+        <v>2026</v>
       </c>
       <c r="J251" t="str">
         <v>Current</v>
@@ -8466,10 +8466,10 @@
         <v>1215.75</v>
       </c>
       <c r="H252" t="str">
-        <v>2025-06-01</v>
+        <v>2025</v>
       </c>
       <c r="I252" t="str">
-        <v>2026-06-31</v>
+        <v>2026</v>
       </c>
       <c r="J252" t="str">
         <v>Current</v>
@@ -8498,10 +8498,10 @@
         <v>1277.25</v>
       </c>
       <c r="H253" t="str">
-        <v>2025-08-01</v>
+        <v>2025</v>
       </c>
       <c r="I253" t="str">
-        <v>2026-08-31</v>
+        <v>2026</v>
       </c>
       <c r="J253" t="str">
         <v>Current</v>
@@ -8530,10 +8530,10 @@
         <v>1205.25</v>
       </c>
       <c r="H254" t="str">
-        <v>2025-06-01</v>
+        <v>2025</v>
       </c>
       <c r="I254" t="str">
-        <v>2026-06-31</v>
+        <v>2026</v>
       </c>
       <c r="J254" t="str">
         <v>Current</v>
@@ -8562,10 +8562,10 @@
         <v>1236</v>
       </c>
       <c r="H255" t="str">
-        <v>2025-07-01</v>
+        <v>2025</v>
       </c>
       <c r="I255" t="str">
-        <v>2026-07-31</v>
+        <v>2026</v>
       </c>
       <c r="J255" t="str">
         <v>Current</v>
@@ -8594,10 +8594,10 @@
         <v>1266.75</v>
       </c>
       <c r="H256" t="str">
-        <v>2025-08-01</v>
+        <v>2025</v>
       </c>
       <c r="I256" t="str">
-        <v>2026-08-31</v>
+        <v>2026</v>
       </c>
       <c r="J256" t="str">
         <v>Current</v>
@@ -8626,10 +8626,10 @@
         <v>1297.5</v>
       </c>
       <c r="H257" t="str">
-        <v>2025-09-01</v>
+        <v>2025</v>
       </c>
       <c r="I257" t="str">
-        <v>2026-09-31</v>
+        <v>2026</v>
       </c>
       <c r="J257" t="str">
         <v>Current</v>
@@ -8658,10 +8658,10 @@
         <v>1205.25</v>
       </c>
       <c r="H258" t="str">
-        <v>2025-06-01</v>
+        <v>2025</v>
       </c>
       <c r="I258" t="str">
-        <v>2026-06-31</v>
+        <v>2026</v>
       </c>
       <c r="J258" t="str">
         <v>Current</v>
@@ -8690,10 +8690,10 @@
         <v>1236</v>
       </c>
       <c r="H259" t="str">
-        <v>2025-07-01</v>
+        <v>2025</v>
       </c>
       <c r="I259" t="str">
-        <v>2026-07-31</v>
+        <v>2026</v>
       </c>
       <c r="J259" t="str">
         <v>Current</v>
@@ -8722,10 +8722,10 @@
         <v>1297.5</v>
       </c>
       <c r="H260" t="str">
-        <v>2025-09-01</v>
+        <v>2025</v>
       </c>
       <c r="I260" t="str">
-        <v>2026-09-31</v>
+        <v>2026</v>
       </c>
       <c r="J260" t="str">
         <v>Current</v>
@@ -8754,10 +8754,10 @@
         <v>1328.25</v>
       </c>
       <c r="H261" t="str">
-        <v>2025-10-01</v>
+        <v>2025</v>
       </c>
       <c r="I261" t="str">
-        <v>2026-10-31</v>
+        <v>2026</v>
       </c>
       <c r="J261" t="str">
         <v>Current</v>
@@ -8786,10 +8786,10 @@
         <v>1205.25</v>
       </c>
       <c r="H262" t="str">
-        <v>2025-06-01</v>
+        <v>2025</v>
       </c>
       <c r="I262" t="str">
-        <v>2026-06-31</v>
+        <v>2026</v>
       </c>
       <c r="J262" t="str">
         <v>Current</v>
@@ -8818,10 +8818,10 @@
         <v>1236</v>
       </c>
       <c r="H263" t="str">
-        <v>2025-07-01</v>
+        <v>2025</v>
       </c>
       <c r="I263" t="str">
-        <v>2026-07-31</v>
+        <v>2026</v>
       </c>
       <c r="J263" t="str">
         <v>Current</v>
@@ -8850,10 +8850,10 @@
         <v>1266.75</v>
       </c>
       <c r="H264" t="str">
-        <v>2025-08-01</v>
+        <v>2025</v>
       </c>
       <c r="I264" t="str">
-        <v>2026-08-31</v>
+        <v>2026</v>
       </c>
       <c r="J264" t="str">
         <v>Current</v>
@@ -8882,10 +8882,10 @@
         <v>1205.25</v>
       </c>
       <c r="H265" t="str">
-        <v>2025-06-01</v>
+        <v>2025</v>
       </c>
       <c r="I265" t="str">
-        <v>2026-06-31</v>
+        <v>2026</v>
       </c>
       <c r="J265" t="str">
         <v>Current</v>
@@ -8914,10 +8914,10 @@
         <v>1236</v>
       </c>
       <c r="H266" t="str">
-        <v>2025-07-01</v>
+        <v>2025</v>
       </c>
       <c r="I266" t="str">
-        <v>2026-07-31</v>
+        <v>2026</v>
       </c>
       <c r="J266" t="str">
         <v>Notice</v>
@@ -8946,10 +8946,10 @@
         <v>1266.75</v>
       </c>
       <c r="H267" t="str">
-        <v>2025-08-01</v>
+        <v>2025</v>
       </c>
       <c r="I267" t="str">
-        <v>2026-08-31</v>
+        <v>2026</v>
       </c>
       <c r="J267" t="str">
         <v>Current</v>
@@ -8978,10 +8978,10 @@
         <v>1205.25</v>
       </c>
       <c r="H268" t="str">
-        <v>2025-06-01</v>
+        <v>2025</v>
       </c>
       <c r="I268" t="str">
-        <v>2026-06-31</v>
+        <v>2026</v>
       </c>
       <c r="J268" t="str">
         <v>Current</v>
@@ -9010,10 +9010,10 @@
         <v>1236</v>
       </c>
       <c r="H269" t="str">
-        <v>2025-07-01</v>
+        <v>2025</v>
       </c>
       <c r="I269" t="str">
-        <v>2026-07-31</v>
+        <v>2026</v>
       </c>
       <c r="J269" t="str">
         <v>Current</v>
@@ -9042,10 +9042,10 @@
         <v>1297.5</v>
       </c>
       <c r="H270" t="str">
-        <v>2025-09-01</v>
+        <v>2025</v>
       </c>
       <c r="I270" t="str">
-        <v>2026-09-31</v>
+        <v>2026</v>
       </c>
       <c r="J270" t="str">
         <v>Current</v>
@@ -9074,10 +9074,10 @@
         <v>1328.25</v>
       </c>
       <c r="H271" t="str">
-        <v>2025-10-01</v>
+        <v>2025</v>
       </c>
       <c r="I271" t="str">
-        <v>2026-10-31</v>
+        <v>2026</v>
       </c>
       <c r="J271" t="str">
         <v>Current</v>
@@ -9106,10 +9106,10 @@
         <v>1205.25</v>
       </c>
       <c r="H272" t="str">
-        <v>2025-06-01</v>
+        <v>2025</v>
       </c>
       <c r="I272" t="str">
-        <v>2026-06-31</v>
+        <v>2026</v>
       </c>
       <c r="J272" t="str">
         <v>Current</v>
@@ -9138,10 +9138,10 @@
         <v>1236</v>
       </c>
       <c r="H273" t="str">
-        <v>2025-07-01</v>
+        <v>2025</v>
       </c>
       <c r="I273" t="str">
-        <v>2026-07-31</v>
+        <v>2026</v>
       </c>
       <c r="J273" t="str">
         <v>Current</v>
@@ -9170,10 +9170,10 @@
         <v>1266.75</v>
       </c>
       <c r="H274" t="str">
-        <v>2025-08-01</v>
+        <v>2025</v>
       </c>
       <c r="I274" t="str">
-        <v>2026-08-31</v>
+        <v>2026</v>
       </c>
       <c r="J274" t="str">
         <v>Current</v>
@@ -9202,10 +9202,10 @@
         <v>1297.5</v>
       </c>
       <c r="H275" t="str">
-        <v>2025-09-01</v>
+        <v>2025</v>
       </c>
       <c r="I275" t="str">
-        <v>2026-09-31</v>
+        <v>2026</v>
       </c>
       <c r="J275" t="str">
         <v>Current</v>
@@ -9234,10 +9234,10 @@
         <v>1225.5</v>
       </c>
       <c r="H276" t="str">
-        <v>2025-07-01</v>
+        <v>2025</v>
       </c>
       <c r="I276" t="str">
-        <v>2026-07-31</v>
+        <v>2026</v>
       </c>
       <c r="J276" t="str">
         <v>Current</v>
@@ -9266,10 +9266,10 @@
         <v>1256.25</v>
       </c>
       <c r="H277" t="str">
-        <v>2025-08-01</v>
+        <v>2025</v>
       </c>
       <c r="I277" t="str">
-        <v>2026-08-31</v>
+        <v>2026</v>
       </c>
       <c r="J277" t="str">
         <v>Current</v>
@@ -9298,10 +9298,10 @@
         <v>1317.75</v>
       </c>
       <c r="H278" t="str">
-        <v>2025-10-01</v>
+        <v>2025</v>
       </c>
       <c r="I278" t="str">
-        <v>2026-10-31</v>
+        <v>2026</v>
       </c>
       <c r="J278" t="str">
         <v>Current</v>
@@ -9330,10 +9330,10 @@
         <v>1225.5</v>
       </c>
       <c r="H279" t="str">
-        <v>2025-07-01</v>
+        <v>2025</v>
       </c>
       <c r="I279" t="str">
-        <v>2026-07-31</v>
+        <v>2026</v>
       </c>
       <c r="J279" t="str">
         <v>Current</v>
@@ -9362,10 +9362,10 @@
         <v>1256.25</v>
       </c>
       <c r="H280" t="str">
-        <v>2025-08-01</v>
+        <v>2025</v>
       </c>
       <c r="I280" t="str">
-        <v>2026-08-31</v>
+        <v>2026</v>
       </c>
       <c r="J280" t="str">
         <v>Current</v>
@@ -9394,10 +9394,10 @@
         <v>1287</v>
       </c>
       <c r="H281" t="str">
-        <v>2025-09-01</v>
+        <v>2025</v>
       </c>
       <c r="I281" t="str">
-        <v>2026-09-31</v>
+        <v>2026</v>
       </c>
       <c r="J281" t="str">
         <v>Current</v>
@@ -9426,10 +9426,10 @@
         <v>1317.75</v>
       </c>
       <c r="H282" t="str">
-        <v>2025-10-01</v>
+        <v>2025</v>
       </c>
       <c r="I282" t="str">
-        <v>2026-10-31</v>
+        <v>2026</v>
       </c>
       <c r="J282" t="str">
         <v>Current</v>
@@ -9458,10 +9458,10 @@
         <v>1348.5</v>
       </c>
       <c r="H283" t="str">
-        <v>2025-11-01</v>
+        <v>2025</v>
       </c>
       <c r="I283" t="str">
-        <v>2026-11-31</v>
+        <v>2026</v>
       </c>
       <c r="J283" t="str">
         <v>Current</v>
@@ -9490,10 +9490,10 @@
         <v>1225.5</v>
       </c>
       <c r="H284" t="str">
-        <v>2025-07-01</v>
+        <v>2025</v>
       </c>
       <c r="I284" t="str">
-        <v>2026-07-31</v>
+        <v>2026</v>
       </c>
       <c r="J284" t="str">
         <v>Current</v>
@@ -9522,10 +9522,10 @@
         <v>1256.25</v>
       </c>
       <c r="H285" t="str">
-        <v>2025-08-01</v>
+        <v>2025</v>
       </c>
       <c r="I285" t="str">
-        <v>2026-08-31</v>
+        <v>2026</v>
       </c>
       <c r="J285" t="str">
         <v>Current</v>
@@ -9554,10 +9554,10 @@
         <v>1225.5</v>
       </c>
       <c r="H286" t="str">
-        <v>2025-07-01</v>
+        <v>2025</v>
       </c>
       <c r="I286" t="str">
-        <v>2026-07-31</v>
+        <v>2026</v>
       </c>
       <c r="J286" t="str">
         <v>Current</v>
@@ -9586,10 +9586,10 @@
         <v>1256.25</v>
       </c>
       <c r="H287" t="str">
-        <v>2025-08-01</v>
+        <v>2025</v>
       </c>
       <c r="I287" t="str">
-        <v>2026-08-31</v>
+        <v>2026</v>
       </c>
       <c r="J287" t="str">
         <v>Current</v>
@@ -9618,10 +9618,10 @@
         <v>1287</v>
       </c>
       <c r="H288" t="str">
-        <v>2025-09-01</v>
+        <v>2025</v>
       </c>
       <c r="I288" t="str">
-        <v>2026-09-31</v>
+        <v>2026</v>
       </c>
       <c r="J288" t="str">
         <v>Current</v>
@@ -9650,10 +9650,10 @@
         <v>1317.75</v>
       </c>
       <c r="H289" t="str">
-        <v>2025-10-01</v>
+        <v>2025</v>
       </c>
       <c r="I289" t="str">
-        <v>2026-10-31</v>
+        <v>2026</v>
       </c>
       <c r="J289" t="str">
         <v>Current</v>
@@ -9682,10 +9682,10 @@
         <v>1348.5</v>
       </c>
       <c r="H290" t="str">
-        <v>2025-11-01</v>
+        <v>2025</v>
       </c>
       <c r="I290" t="str">
-        <v>2026-11-31</v>
+        <v>2026</v>
       </c>
       <c r="J290" t="str">
         <v>Current</v>
@@ -9714,10 +9714,10 @@
         <v>1225.5</v>
       </c>
       <c r="H291" t="str">
-        <v>2025-07-01</v>
+        <v>2025</v>
       </c>
       <c r="I291" t="str">
-        <v>2026-07-31</v>
+        <v>2026</v>
       </c>
       <c r="J291" t="str">
         <v>Current</v>
@@ -9746,10 +9746,10 @@
         <v>1256.25</v>
       </c>
       <c r="H292" t="str">
-        <v>2025-08-01</v>
+        <v>2025</v>
       </c>
       <c r="I292" t="str">
-        <v>2026-08-31</v>
+        <v>2026</v>
       </c>
       <c r="J292" t="str">
         <v>Current</v>
@@ -9778,10 +9778,10 @@
         <v>1287</v>
       </c>
       <c r="H293" t="str">
-        <v>2025-09-01</v>
+        <v>2025</v>
       </c>
       <c r="I293" t="str">
-        <v>2026-09-31</v>
+        <v>2026</v>
       </c>
       <c r="J293" t="str">
         <v>Current</v>
@@ -9810,10 +9810,10 @@
         <v>1317.75</v>
       </c>
       <c r="H294" t="str">
-        <v>2025-10-01</v>
+        <v>2025</v>
       </c>
       <c r="I294" t="str">
-        <v>2026-10-31</v>
+        <v>2026</v>
       </c>
       <c r="J294" t="str">
         <v>Current</v>
@@ -9842,10 +9842,10 @@
         <v>1245.75</v>
       </c>
       <c r="H295" t="str">
-        <v>2025-08-01</v>
+        <v>2025</v>
       </c>
       <c r="I295" t="str">
-        <v>2026-08-31</v>
+        <v>2026</v>
       </c>
       <c r="J295" t="str">
         <v>Current</v>
@@ -9874,10 +9874,10 @@
         <v>1276.5</v>
       </c>
       <c r="H296" t="str">
-        <v>2025-09-01</v>
+        <v>2025</v>
       </c>
       <c r="I296" t="str">
-        <v>2026-09-31</v>
+        <v>2026</v>
       </c>
       <c r="J296" t="str">
         <v>Current</v>
@@ -9906,10 +9906,10 @@
         <v>1307.25</v>
       </c>
       <c r="H297" t="str">
-        <v>2025-10-01</v>
+        <v>2025</v>
       </c>
       <c r="I297" t="str">
-        <v>2026-10-31</v>
+        <v>2026</v>
       </c>
       <c r="J297" t="str">
         <v>Current</v>
@@ -9938,10 +9938,10 @@
         <v>1338</v>
       </c>
       <c r="H298" t="str">
-        <v>2025-11-01</v>
+        <v>2025</v>
       </c>
       <c r="I298" t="str">
-        <v>2026-11-31</v>
+        <v>2026</v>
       </c>
       <c r="J298" t="str">
         <v>Current</v>
@@ -9970,10 +9970,10 @@
         <v>1245.75</v>
       </c>
       <c r="H299" t="str">
-        <v>2025-08-01</v>
+        <v>2025</v>
       </c>
       <c r="I299" t="str">
-        <v>2026-08-31</v>
+        <v>2026</v>
       </c>
       <c r="J299" t="str">
         <v>Current</v>
@@ -10002,10 +10002,10 @@
         <v>1276.5</v>
       </c>
       <c r="H300" t="str">
-        <v>2025-09-01</v>
+        <v>2025</v>
       </c>
       <c r="I300" t="str">
-        <v>2026-09-31</v>
+        <v>2026</v>
       </c>
       <c r="J300" t="str">
         <v>Notice</v>
@@ -10034,10 +10034,10 @@
         <v>1307.25</v>
       </c>
       <c r="H301" t="str">
-        <v>2025-10-01</v>
+        <v>2025</v>
       </c>
       <c r="I301" t="str">
-        <v>2026-10-31</v>
+        <v>2026</v>
       </c>
       <c r="J301" t="str">
         <v>Current</v>
@@ -10066,10 +10066,10 @@
         <v>1338</v>
       </c>
       <c r="H302" t="str">
-        <v>2025-11-01</v>
+        <v>2025</v>
       </c>
       <c r="I302" t="str">
-        <v>2026-11-31</v>
+        <v>2026</v>
       </c>
       <c r="J302" t="str">
         <v>Current</v>
@@ -10098,10 +10098,10 @@
         <v>1368.75</v>
       </c>
       <c r="H303" t="str">
-        <v>2025-12-01</v>
+        <v>2025</v>
       </c>
       <c r="I303" t="str">
-        <v>2026-12-31</v>
+        <v>2026</v>
       </c>
       <c r="J303" t="str">
         <v>Current</v>
@@ -10130,10 +10130,10 @@
         <v>1245.75</v>
       </c>
       <c r="H304" t="str">
-        <v>2025-08-01</v>
+        <v>2025</v>
       </c>
       <c r="I304" t="str">
-        <v>2026-08-31</v>
+        <v>2026</v>
       </c>
       <c r="J304" t="str">
         <v>Current</v>
@@ -10162,10 +10162,10 @@
         <v>1276.5</v>
       </c>
       <c r="H305" t="str">
-        <v>2025-09-01</v>
+        <v>2025</v>
       </c>
       <c r="I305" t="str">
-        <v>2026-09-31</v>
+        <v>2026</v>
       </c>
       <c r="J305" t="str">
         <v>Current</v>
@@ -10194,10 +10194,10 @@
         <v>1245.75</v>
       </c>
       <c r="H306" t="str">
-        <v>2025-08-01</v>
+        <v>2025</v>
       </c>
       <c r="I306" t="str">
-        <v>2026-08-31</v>
+        <v>2026</v>
       </c>
       <c r="J306" t="str">
         <v>Current</v>
@@ -10226,10 +10226,10 @@
         <v>1276.5</v>
       </c>
       <c r="H307" t="str">
-        <v>2025-09-01</v>
+        <v>2025</v>
       </c>
       <c r="I307" t="str">
-        <v>2026-09-31</v>
+        <v>2026</v>
       </c>
       <c r="J307" t="str">
         <v>Current</v>
@@ -10258,10 +10258,10 @@
         <v>1307.25</v>
       </c>
       <c r="H308" t="str">
-        <v>2025-10-01</v>
+        <v>2025</v>
       </c>
       <c r="I308" t="str">
-        <v>2026-10-31</v>
+        <v>2026</v>
       </c>
       <c r="J308" t="str">
         <v>Current</v>
@@ -10290,10 +10290,10 @@
         <v>1245.75</v>
       </c>
       <c r="H309" t="str">
-        <v>2025-08-01</v>
+        <v>2025</v>
       </c>
       <c r="I309" t="str">
-        <v>2026-08-31</v>
+        <v>2026</v>
       </c>
       <c r="J309" t="str">
         <v>Current</v>
@@ -10322,10 +10322,10 @@
         <v>1276.5</v>
       </c>
       <c r="H310" t="str">
-        <v>2025-09-01</v>
+        <v>2025</v>
       </c>
       <c r="I310" t="str">
-        <v>2026-09-31</v>
+        <v>2026</v>
       </c>
       <c r="J310" t="str">
         <v>Current</v>
@@ -10354,10 +10354,10 @@
         <v>1307.25</v>
       </c>
       <c r="H311" t="str">
-        <v>2025-10-01</v>
+        <v>2025</v>
       </c>
       <c r="I311" t="str">
-        <v>2026-10-31</v>
+        <v>2026</v>
       </c>
       <c r="J311" t="str">
         <v>Current</v>
@@ -10386,10 +10386,10 @@
         <v>1338</v>
       </c>
       <c r="H312" t="str">
-        <v>2025-11-01</v>
+        <v>2025</v>
       </c>
       <c r="I312" t="str">
-        <v>2026-11-31</v>
+        <v>2026</v>
       </c>
       <c r="J312" t="str">
         <v>Current</v>
@@ -10418,10 +10418,10 @@
         <v>1368.75</v>
       </c>
       <c r="H313" t="str">
-        <v>2025-12-01</v>
+        <v>2025</v>
       </c>
       <c r="I313" t="str">
-        <v>2026-12-31</v>
+        <v>2026</v>
       </c>
       <c r="J313" t="str">
         <v>Current</v>
@@ -10450,10 +10450,10 @@
         <v>1245.75</v>
       </c>
       <c r="H314" t="str">
-        <v>2025-08-01</v>
+        <v>2025</v>
       </c>
       <c r="I314" t="str">
-        <v>2026-08-31</v>
+        <v>2026</v>
       </c>
       <c r="J314" t="str">
         <v>Current</v>
@@ -10482,10 +10482,10 @@
         <v>1276.5</v>
       </c>
       <c r="H315" t="str">
-        <v>2025-09-01</v>
+        <v>2025</v>
       </c>
       <c r="I315" t="str">
-        <v>2026-09-31</v>
+        <v>2026</v>
       </c>
       <c r="J315" t="str">
         <v>Notice</v>
@@ -10514,10 +10514,10 @@
         <v>1338</v>
       </c>
       <c r="H316" t="str">
-        <v>2025-11-01</v>
+        <v>2025</v>
       </c>
       <c r="I316" t="str">
-        <v>2026-11-31</v>
+        <v>2026</v>
       </c>
       <c r="J316" t="str">
         <v>Current</v>
@@ -10546,10 +10546,10 @@
         <v>1266</v>
       </c>
       <c r="H317" t="str">
-        <v>2025-09-01</v>
+        <v>2025</v>
       </c>
       <c r="I317" t="str">
-        <v>2026-09-31</v>
+        <v>2026</v>
       </c>
       <c r="J317" t="str">
         <v>Future</v>
@@ -10578,10 +10578,10 @@
         <v>1296.75</v>
       </c>
       <c r="H318" t="str">
-        <v>2025-10-01</v>
+        <v>2025</v>
       </c>
       <c r="I318" t="str">
-        <v>2026-10-31</v>
+        <v>2026</v>
       </c>
       <c r="J318" t="str">
         <v>Future</v>
@@ -10610,10 +10610,10 @@
         <v>1327.5</v>
       </c>
       <c r="H319" t="str">
-        <v>2025-11-01</v>
+        <v>2025</v>
       </c>
       <c r="I319" t="str">
-        <v>2026-11-31</v>
+        <v>2026</v>
       </c>
       <c r="J319" t="str">
         <v>Future</v>
@@ -10642,10 +10642,10 @@
         <v>1358.25</v>
       </c>
       <c r="H320" t="str">
-        <v>2025-12-01</v>
+        <v>2025</v>
       </c>
       <c r="I320" t="str">
-        <v>2026-12-31</v>
+        <v>2026</v>
       </c>
       <c r="J320" t="str">
         <v>Future</v>
@@ -10674,10 +10674,10 @@
         <v>1266</v>
       </c>
       <c r="H321" t="str">
-        <v>2025-09-01</v>
+        <v>2025</v>
       </c>
       <c r="I321" t="str">
-        <v>2026-09-31</v>
+        <v>2026</v>
       </c>
       <c r="J321" t="str">
         <v>Current</v>
@@ -10706,10 +10706,10 @@
         <v>1296.75</v>
       </c>
       <c r="H322" t="str">
-        <v>2025-10-01</v>
+        <v>2025</v>
       </c>
       <c r="I322" t="str">
-        <v>2026-10-31</v>
+        <v>2026</v>
       </c>
       <c r="J322" t="str">
         <v>Current</v>
@@ -10738,10 +10738,10 @@
         <v>1358.25</v>
       </c>
       <c r="H323" t="str">
-        <v>2025-12-01</v>
+        <v>2025</v>
       </c>
       <c r="I323" t="str">
-        <v>2026-12-31</v>
+        <v>2026</v>
       </c>
       <c r="J323" t="str">
         <v>Current</v>
@@ -10770,10 +10770,10 @@
         <v>1389</v>
       </c>
       <c r="H324" t="str">
-        <v>2025-01-01</v>
+        <v>2025</v>
       </c>
       <c r="I324" t="str">
-        <v>2026-01-31</v>
+        <v>2026</v>
       </c>
       <c r="J324" t="str">
         <v>Current</v>
@@ -10802,10 +10802,10 @@
         <v>1266</v>
       </c>
       <c r="H325" t="str">
-        <v>2025-09-01</v>
+        <v>2025</v>
       </c>
       <c r="I325" t="str">
-        <v>2026-09-31</v>
+        <v>2026</v>
       </c>
       <c r="J325" t="str">
         <v>Current</v>
@@ -10834,10 +10834,10 @@
         <v>1296.75</v>
       </c>
       <c r="H326" t="str">
-        <v>2025-10-01</v>
+        <v>2025</v>
       </c>
       <c r="I326" t="str">
-        <v>2026-10-31</v>
+        <v>2026</v>
       </c>
       <c r="J326" t="str">
         <v>Current</v>
@@ -10866,10 +10866,10 @@
         <v>1327.5</v>
       </c>
       <c r="H327" t="str">
-        <v>2025-11-01</v>
+        <v>2025</v>
       </c>
       <c r="I327" t="str">
-        <v>2026-11-31</v>
+        <v>2026</v>
       </c>
       <c r="J327" t="str">
         <v>Current</v>
@@ -10898,10 +10898,10 @@
         <v>1266</v>
       </c>
       <c r="H328" t="str">
-        <v>2025-09-01</v>
+        <v>2025</v>
       </c>
       <c r="I328" t="str">
-        <v>2026-09-31</v>
+        <v>2026</v>
       </c>
       <c r="J328" t="str">
         <v>Current</v>
@@ -10930,10 +10930,10 @@
         <v>1296.75</v>
       </c>
       <c r="H329" t="str">
-        <v>2025-10-01</v>
+        <v>2025</v>
       </c>
       <c r="I329" t="str">
-        <v>2026-10-31</v>
+        <v>2026</v>
       </c>
       <c r="J329" t="str">
         <v>Current</v>
@@ -10962,10 +10962,10 @@
         <v>1327.5</v>
       </c>
       <c r="H330" t="str">
-        <v>2025-11-01</v>
+        <v>2025</v>
       </c>
       <c r="I330" t="str">
-        <v>2026-11-31</v>
+        <v>2026</v>
       </c>
       <c r="J330" t="str">
         <v>Current</v>
@@ -10994,10 +10994,10 @@
         <v>1266</v>
       </c>
       <c r="H331" t="str">
-        <v>2025-09-01</v>
+        <v>2025</v>
       </c>
       <c r="I331" t="str">
-        <v>2026-09-31</v>
+        <v>2026</v>
       </c>
       <c r="J331" t="str">
         <v>Current</v>
@@ -11026,10 +11026,10 @@
         <v>1296.75</v>
       </c>
       <c r="H332" t="str">
-        <v>2025-10-01</v>
+        <v>2025</v>
       </c>
       <c r="I332" t="str">
-        <v>2026-10-31</v>
+        <v>2026</v>
       </c>
       <c r="J332" t="str">
         <v>Notice</v>
@@ -11058,10 +11058,10 @@
         <v>1358.25</v>
       </c>
       <c r="H333" t="str">
-        <v>2025-12-01</v>
+        <v>2025</v>
       </c>
       <c r="I333" t="str">
-        <v>2026-12-31</v>
+        <v>2026</v>
       </c>
       <c r="J333" t="str">
         <v>Current</v>
@@ -11090,10 +11090,10 @@
         <v>1389</v>
       </c>
       <c r="H334" t="str">
-        <v>2025-01-01</v>
+        <v>2025</v>
       </c>
       <c r="I334" t="str">
-        <v>2026-01-31</v>
+        <v>2026</v>
       </c>
       <c r="J334" t="str">
         <v>Current</v>
@@ -11122,10 +11122,10 @@
         <v>1266</v>
       </c>
       <c r="H335" t="str">
-        <v>2025-09-01</v>
+        <v>2025</v>
       </c>
       <c r="I335" t="str">
-        <v>2026-09-31</v>
+        <v>2026</v>
       </c>
       <c r="J335" t="str">
         <v>Current</v>
@@ -11154,10 +11154,10 @@
         <v>1296.75</v>
       </c>
       <c r="H336" t="str">
-        <v>2025-10-01</v>
+        <v>2025</v>
       </c>
       <c r="I336" t="str">
-        <v>2026-10-31</v>
+        <v>2026</v>
       </c>
       <c r="J336" t="str">
         <v>Current</v>
@@ -11186,10 +11186,10 @@
         <v>1327.5</v>
       </c>
       <c r="H337" t="str">
-        <v>2025-11-01</v>
+        <v>2025</v>
       </c>
       <c r="I337" t="str">
-        <v>2026-11-31</v>
+        <v>2026</v>
       </c>
       <c r="J337" t="str">
         <v>Current</v>
@@ -11218,10 +11218,10 @@
         <v>1358.25</v>
       </c>
       <c r="H338" t="str">
-        <v>2025-12-01</v>
+        <v>2025</v>
       </c>
       <c r="I338" t="str">
-        <v>2026-12-31</v>
+        <v>2026</v>
       </c>
       <c r="J338" t="str">
         <v>Current</v>
@@ -11250,10 +11250,10 @@
         <v>1286.25</v>
       </c>
       <c r="H339" t="str">
-        <v>2025-10-01</v>
+        <v>2025</v>
       </c>
       <c r="I339" t="str">
-        <v>2026-10-31</v>
+        <v>2026</v>
       </c>
       <c r="J339" t="str">
         <v>Current</v>
@@ -11282,10 +11282,10 @@
         <v>1317</v>
       </c>
       <c r="H340" t="str">
-        <v>2025-11-01</v>
+        <v>2025</v>
       </c>
       <c r="I340" t="str">
-        <v>2026-11-31</v>
+        <v>2026</v>
       </c>
       <c r="J340" t="str">
         <v>Current</v>
@@ -11314,10 +11314,10 @@
         <v>1378.5</v>
       </c>
       <c r="H341" t="str">
-        <v>2025-01-01</v>
+        <v>2025</v>
       </c>
       <c r="I341" t="str">
-        <v>2026-01-31</v>
+        <v>2026</v>
       </c>
       <c r="J341" t="str">
         <v>Current</v>
@@ -11346,10 +11346,10 @@
         <v>1286.25</v>
       </c>
       <c r="H342" t="str">
-        <v>2025-10-01</v>
+        <v>2025</v>
       </c>
       <c r="I342" t="str">
-        <v>2026-10-31</v>
+        <v>2026</v>
       </c>
       <c r="J342" t="str">
         <v>Current</v>
@@ -11378,10 +11378,10 @@
         <v>1317</v>
       </c>
       <c r="H343" t="str">
-        <v>2025-11-01</v>
+        <v>2025</v>
       </c>
       <c r="I343" t="str">
-        <v>2026-11-31</v>
+        <v>2026</v>
       </c>
       <c r="J343" t="str">
         <v>Current</v>
@@ -11410,10 +11410,10 @@
         <v>1347.75</v>
       </c>
       <c r="H344" t="str">
-        <v>2025-12-01</v>
+        <v>2025</v>
       </c>
       <c r="I344" t="str">
-        <v>2026-12-31</v>
+        <v>2026</v>
       </c>
       <c r="J344" t="str">
         <v>Current</v>
@@ -11442,10 +11442,10 @@
         <v>1378.5</v>
       </c>
       <c r="H345" t="str">
-        <v>2025-01-01</v>
+        <v>2025</v>
       </c>
       <c r="I345" t="str">
-        <v>2026-01-31</v>
+        <v>2026</v>
       </c>
       <c r="J345" t="str">
         <v>Current</v>
@@ -11474,10 +11474,10 @@
         <v>1409.25</v>
       </c>
       <c r="H346" t="str">
-        <v>2025-02-01</v>
+        <v>2025</v>
       </c>
       <c r="I346" t="str">
-        <v>2026-02-31</v>
+        <v>2026</v>
       </c>
       <c r="J346" t="str">
         <v>Current</v>
@@ -11506,10 +11506,10 @@
         <v>1286.25</v>
       </c>
       <c r="H347" t="str">
-        <v>2025-10-01</v>
+        <v>2025</v>
       </c>
       <c r="I347" t="str">
-        <v>2026-10-31</v>
+        <v>2026</v>
       </c>
       <c r="J347" t="str">
         <v>Current</v>
@@ -11538,10 +11538,10 @@
         <v>1317</v>
       </c>
       <c r="H348" t="str">
-        <v>2025-11-01</v>
+        <v>2025</v>
       </c>
       <c r="I348" t="str">
-        <v>2026-11-31</v>
+        <v>2026</v>
       </c>
       <c r="J348" t="str">
         <v>Current</v>
@@ -11570,10 +11570,10 @@
         <v>1347.75</v>
       </c>
       <c r="H349" t="str">
-        <v>2025-12-01</v>
+        <v>2025</v>
       </c>
       <c r="I349" t="str">
-        <v>2026-12-31</v>
+        <v>2026</v>
       </c>
       <c r="J349" t="str">
         <v>Current</v>
@@ -11602,10 +11602,10 @@
         <v>1286.25</v>
       </c>
       <c r="H350" t="str">
-        <v>2025-10-01</v>
+        <v>2025</v>
       </c>
       <c r="I350" t="str">
-        <v>2026-10-31</v>
+        <v>2026</v>
       </c>
       <c r="J350" t="str">
         <v>Current</v>
@@ -11634,10 +11634,10 @@
         <v>1317</v>
       </c>
       <c r="H351" t="str">
-        <v>2025-11-01</v>
+        <v>2025</v>
       </c>
       <c r="I351" t="str">
-        <v>2026-11-31</v>
+        <v>2026</v>
       </c>
       <c r="J351" t="str">
         <v>Notice</v>
@@ -11666,10 +11666,10 @@
         <v>1286.25</v>
       </c>
       <c r="H352" t="str">
-        <v>2025-10-01</v>
+        <v>2025</v>
       </c>
       <c r="I352" t="str">
-        <v>2026-10-31</v>
+        <v>2026</v>
       </c>
       <c r="J352" t="str">
         <v>Current</v>
@@ -11698,10 +11698,10 @@
         <v>1317</v>
       </c>
       <c r="H353" t="str">
-        <v>2025-11-01</v>
+        <v>2025</v>
       </c>
       <c r="I353" t="str">
-        <v>2026-11-31</v>
+        <v>2026</v>
       </c>
       <c r="J353" t="str">
         <v>Current</v>
@@ -11730,10 +11730,10 @@
         <v>1347.75</v>
       </c>
       <c r="H354" t="str">
-        <v>2025-12-01</v>
+        <v>2025</v>
       </c>
       <c r="I354" t="str">
-        <v>2026-12-31</v>
+        <v>2026</v>
       </c>
       <c r="J354" t="str">
         <v>Current</v>
@@ -11762,10 +11762,10 @@
         <v>1378.5</v>
       </c>
       <c r="H355" t="str">
-        <v>2025-01-01</v>
+        <v>2025</v>
       </c>
       <c r="I355" t="str">
-        <v>2026-01-31</v>
+        <v>2026</v>
       </c>
       <c r="J355" t="str">
         <v>Current</v>
@@ -11794,10 +11794,10 @@
         <v>1409.25</v>
       </c>
       <c r="H356" t="str">
-        <v>2025-02-01</v>
+        <v>2025</v>
       </c>
       <c r="I356" t="str">
-        <v>2026-02-31</v>
+        <v>2026</v>
       </c>
       <c r="J356" t="str">
         <v>Current</v>
@@ -11826,10 +11826,10 @@
         <v>1306.5</v>
       </c>
       <c r="H357" t="str">
-        <v>2025-11-01</v>
+        <v>2025</v>
       </c>
       <c r="I357" t="str">
-        <v>2026-11-31</v>
+        <v>2026</v>
       </c>
       <c r="J357" t="str">
         <v>Current</v>
@@ -11858,10 +11858,10 @@
         <v>1337.25</v>
       </c>
       <c r="H358" t="str">
-        <v>2025-12-01</v>
+        <v>2025</v>
       </c>
       <c r="I358" t="str">
-        <v>2026-12-31</v>
+        <v>2026</v>
       </c>
       <c r="J358" t="str">
         <v>Current</v>
@@ -11890,10 +11890,10 @@
         <v>1368</v>
       </c>
       <c r="H359" t="str">
-        <v>2025-01-01</v>
+        <v>2025</v>
       </c>
       <c r="I359" t="str">
-        <v>2026-01-31</v>
+        <v>2026</v>
       </c>
       <c r="J359" t="str">
         <v>Current</v>
@@ -11922,10 +11922,10 @@
         <v>1398.75</v>
       </c>
       <c r="H360" t="str">
-        <v>2025-02-01</v>
+        <v>2025</v>
       </c>
       <c r="I360" t="str">
-        <v>2026-02-31</v>
+        <v>2026</v>
       </c>
       <c r="J360" t="str">
         <v>Current</v>
@@ -11954,10 +11954,10 @@
         <v>1306.5</v>
       </c>
       <c r="H361" t="str">
-        <v>2025-11-01</v>
+        <v>2025</v>
       </c>
       <c r="I361" t="str">
-        <v>2026-11-31</v>
+        <v>2026</v>
       </c>
       <c r="J361" t="str">
         <v>Current</v>
@@ -11986,10 +11986,10 @@
         <v>1337.25</v>
       </c>
       <c r="H362" t="str">
-        <v>2025-12-01</v>
+        <v>2025</v>
       </c>
       <c r="I362" t="str">
-        <v>2026-12-31</v>
+        <v>2026</v>
       </c>
       <c r="J362" t="str">
         <v>Current</v>
@@ -12018,10 +12018,10 @@
         <v>1368</v>
       </c>
       <c r="H363" t="str">
-        <v>2025-01-01</v>
+        <v>2025</v>
       </c>
       <c r="I363" t="str">
-        <v>2026-01-31</v>
+        <v>2026</v>
       </c>
       <c r="J363" t="str">
         <v>Current</v>
@@ -12050,10 +12050,10 @@
         <v>1398.75</v>
       </c>
       <c r="H364" t="str">
-        <v>2025-02-01</v>
+        <v>2025</v>
       </c>
       <c r="I364" t="str">
-        <v>2026-02-31</v>
+        <v>2026</v>
       </c>
       <c r="J364" t="str">
         <v>Current</v>
@@ -12082,10 +12082,10 @@
         <v>1429.5</v>
       </c>
       <c r="H365" t="str">
-        <v>2025-03-01</v>
+        <v>2025</v>
       </c>
       <c r="I365" t="str">
-        <v>2026-03-31</v>
+        <v>2026</v>
       </c>
       <c r="J365" t="str">
         <v>Current</v>
@@ -12114,10 +12114,10 @@
         <v>1306.5</v>
       </c>
       <c r="H366" t="str">
-        <v>2025-11-01</v>
+        <v>2025</v>
       </c>
       <c r="I366" t="str">
-        <v>2026-11-31</v>
+        <v>2026</v>
       </c>
       <c r="J366" t="str">
         <v>Current</v>
@@ -12146,10 +12146,10 @@
         <v>1337.25</v>
       </c>
       <c r="H367" t="str">
-        <v>2025-12-01</v>
+        <v>2025</v>
       </c>
       <c r="I367" t="str">
-        <v>2026-12-31</v>
+        <v>2026</v>
       </c>
       <c r="J367" t="str">
         <v>Notice</v>
@@ -12178,10 +12178,10 @@
         <v>1306.5</v>
       </c>
       <c r="H368" t="str">
-        <v>2025-11-01</v>
+        <v>2025</v>
       </c>
       <c r="I368" t="str">
-        <v>2026-11-31</v>
+        <v>2026</v>
       </c>
       <c r="J368" t="str">
         <v>Current</v>
@@ -12210,10 +12210,10 @@
         <v>1337.25</v>
       </c>
       <c r="H369" t="str">
-        <v>2025-12-01</v>
+        <v>2025</v>
       </c>
       <c r="I369" t="str">
-        <v>2026-12-31</v>
+        <v>2026</v>
       </c>
       <c r="J369" t="str">
         <v>Current</v>
@@ -12242,10 +12242,10 @@
         <v>1368</v>
       </c>
       <c r="H370" t="str">
-        <v>2025-01-01</v>
+        <v>2025</v>
       </c>
       <c r="I370" t="str">
-        <v>2026-01-31</v>
+        <v>2026</v>
       </c>
       <c r="J370" t="str">
         <v>Current</v>
@@ -12274,10 +12274,10 @@
         <v>1306.5</v>
       </c>
       <c r="H371" t="str">
-        <v>2025-11-01</v>
+        <v>2025</v>
       </c>
       <c r="I371" t="str">
-        <v>2026-11-31</v>
+        <v>2026</v>
       </c>
       <c r="J371" t="str">
         <v>Current</v>
@@ -12306,10 +12306,10 @@
         <v>1337.25</v>
       </c>
       <c r="H372" t="str">
-        <v>2025-12-01</v>
+        <v>2025</v>
       </c>
       <c r="I372" t="str">
-        <v>2026-12-31</v>
+        <v>2026</v>
       </c>
       <c r="J372" t="str">
         <v>Current</v>
@@ -12338,10 +12338,10 @@
         <v>1368</v>
       </c>
       <c r="H373" t="str">
-        <v>2025-01-01</v>
+        <v>2025</v>
       </c>
       <c r="I373" t="str">
-        <v>2026-01-31</v>
+        <v>2026</v>
       </c>
       <c r="J373" t="str">
         <v>Current</v>
@@ -12370,10 +12370,10 @@
         <v>1398.75</v>
       </c>
       <c r="H374" t="str">
-        <v>2025-02-01</v>
+        <v>2025</v>
       </c>
       <c r="I374" t="str">
-        <v>2026-02-31</v>
+        <v>2026</v>
       </c>
       <c r="J374" t="str">
         <v>Current</v>
@@ -12402,10 +12402,10 @@
         <v>1429.5</v>
       </c>
       <c r="H375" t="str">
-        <v>2025-03-01</v>
+        <v>2025</v>
       </c>
       <c r="I375" t="str">
-        <v>2026-03-31</v>
+        <v>2026</v>
       </c>
       <c r="J375" t="str">
         <v>Current</v>
@@ -12434,10 +12434,10 @@
         <v>1306.5</v>
       </c>
       <c r="H376" t="str">
-        <v>2025-11-01</v>
+        <v>2025</v>
       </c>
       <c r="I376" t="str">
-        <v>2026-11-31</v>
+        <v>2026</v>
       </c>
       <c r="J376" t="str">
         <v>Current</v>
@@ -12466,10 +12466,10 @@
         <v>1337.25</v>
       </c>
       <c r="H377" t="str">
-        <v>2025-12-01</v>
+        <v>2025</v>
       </c>
       <c r="I377" t="str">
-        <v>2026-12-31</v>
+        <v>2026</v>
       </c>
       <c r="J377" t="str">
         <v>Current</v>
@@ -12498,10 +12498,10 @@
         <v>1398.75</v>
       </c>
       <c r="H378" t="str">
-        <v>2025-02-01</v>
+        <v>2025</v>
       </c>
       <c r="I378" t="str">
-        <v>2026-02-31</v>
+        <v>2026</v>
       </c>
       <c r="J378" t="str">
         <v>Current</v>

</xml_diff>